<commit_message>
finished update of explosive production
</commit_message>
<xml_diff>
--- a/gui/rebalance_localizations.xlsx
+++ b/gui/rebalance_localizations.xlsx
@@ -16,14 +16,14 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">rebalance_localizations!$A$1:$K$920</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">rebalance_localizations!$A$1:$K$921</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="1737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1925" uniqueCount="1739">
   <si>
     <t>ENGLISH</t>
   </si>
@@ -5234,6 +5234,12 @@
   </si>
   <si>
     <t>Reagent Well</t>
+  </si>
+  <si>
+    <t>Advanced Nuclear Explosives</t>
+  </si>
+  <si>
+    <t>gui/menu/research/name/ammo_explosive_fissonium</t>
   </si>
 </sst>
 </file>
@@ -6077,7 +6083,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K920"/>
+  <dimension ref="A1:K921"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="65.453125" customWidth="1"/>
@@ -11119,47 +11125,47 @@
     </row>
     <row r="622" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A622" t="s">
-        <v>1538</v>
+        <v>1738</v>
       </c>
       <c r="B622" s="1" t="s">
-        <v>1541</v>
+        <v>1737</v>
       </c>
     </row>
     <row r="623" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A623" t="s">
-        <v>498</v>
+        <v>1538</v>
       </c>
       <c r="B623" s="1" t="s">
-        <v>519</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="624" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A624" t="s">
-        <v>1173</v>
+        <v>498</v>
       </c>
       <c r="B624" s="1" t="s">
-        <v>1144</v>
+        <v>519</v>
       </c>
     </row>
     <row r="625" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A625" t="s">
-        <v>499</v>
+        <v>1173</v>
       </c>
       <c r="B625" s="1" t="s">
-        <v>649</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="626" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A626" t="s">
-        <v>646</v>
+        <v>499</v>
       </c>
       <c r="B626" s="1" t="s">
-        <v>1145</v>
+        <v>649</v>
       </c>
     </row>
     <row r="627" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A627" t="s">
-        <v>1587</v>
+        <v>646</v>
       </c>
       <c r="B627" s="1" t="s">
         <v>1145</v>
@@ -11167,39 +11173,39 @@
     </row>
     <row r="628" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A628" t="s">
-        <v>500</v>
+        <v>1587</v>
       </c>
       <c r="B628" s="1" t="s">
-        <v>517</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="629" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A629" t="s">
-        <v>1174</v>
+        <v>500</v>
       </c>
       <c r="B629" s="1" t="s">
-        <v>1139</v>
+        <v>517</v>
       </c>
     </row>
     <row r="630" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A630" t="s">
-        <v>501</v>
+        <v>1174</v>
       </c>
       <c r="B630" s="1" t="s">
-        <v>650</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="631" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A631" t="s">
-        <v>645</v>
+        <v>501</v>
       </c>
       <c r="B631" s="1" t="s">
-        <v>1142</v>
+        <v>650</v>
       </c>
     </row>
     <row r="632" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A632" t="s">
-        <v>1588</v>
+        <v>645</v>
       </c>
       <c r="B632" s="1" t="s">
         <v>1142</v>
@@ -11207,39 +11213,39 @@
     </row>
     <row r="633" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A633" t="s">
-        <v>502</v>
+        <v>1588</v>
       </c>
       <c r="B633" s="1" t="s">
-        <v>520</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="634" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A634" t="s">
-        <v>1175</v>
+        <v>502</v>
       </c>
       <c r="B634" s="1" t="s">
-        <v>1146</v>
+        <v>520</v>
       </c>
     </row>
     <row r="635" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A635" t="s">
-        <v>503</v>
+        <v>1175</v>
       </c>
       <c r="B635" s="1" t="s">
-        <v>651</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="636" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A636" t="s">
-        <v>644</v>
+        <v>503</v>
       </c>
       <c r="B636" s="1" t="s">
-        <v>1147</v>
+        <v>651</v>
       </c>
     </row>
     <row r="637" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A637" t="s">
-        <v>1589</v>
+        <v>644</v>
       </c>
       <c r="B637" s="1" t="s">
         <v>1147</v>
@@ -11247,39 +11253,39 @@
     </row>
     <row r="638" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A638" t="s">
-        <v>504</v>
+        <v>1589</v>
       </c>
       <c r="B638" s="1" t="s">
-        <v>518</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="639" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A639" t="s">
-        <v>1176</v>
+        <v>504</v>
       </c>
       <c r="B639" s="1" t="s">
-        <v>1140</v>
+        <v>518</v>
       </c>
     </row>
     <row r="640" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A640" t="s">
-        <v>505</v>
+        <v>1176</v>
       </c>
       <c r="B640" s="1" t="s">
-        <v>652</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="641" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A641" t="s">
-        <v>643</v>
+        <v>505</v>
       </c>
       <c r="B641" s="1" t="s">
-        <v>1143</v>
+        <v>652</v>
       </c>
     </row>
     <row r="642" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A642" t="s">
-        <v>1590</v>
+        <v>643</v>
       </c>
       <c r="B642" s="1" t="s">
         <v>1143</v>
@@ -11287,554 +11293,554 @@
     </row>
     <row r="643" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A643" t="s">
-        <v>1539</v>
+        <v>1590</v>
       </c>
       <c r="B643" s="1" t="s">
-        <v>1540</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="644" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A644" t="s">
-        <v>1017</v>
+        <v>1539</v>
       </c>
       <c r="B644" s="1" t="s">
-        <v>1020</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="645" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A645" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="B645" s="1" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="646" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A646" t="s">
-        <v>1005</v>
+        <v>1016</v>
       </c>
       <c r="B646" s="1" t="s">
-        <v>1014</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="647" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A647" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B647" s="1" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="648" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A648" t="s">
-        <v>169</v>
+        <v>1006</v>
       </c>
       <c r="B648" s="1" t="s">
-        <v>170</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="649" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A649" t="s">
-        <v>1177</v>
+        <v>169</v>
       </c>
       <c r="B649" s="1" t="s">
-        <v>1185</v>
+        <v>170</v>
       </c>
     </row>
     <row r="650" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
-        <v>1193</v>
+        <v>1177</v>
       </c>
       <c r="B650" s="1" t="s">
-        <v>1201</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="651" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
-        <v>171</v>
+        <v>1193</v>
       </c>
       <c r="B651" s="1" t="s">
-        <v>172</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="652" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
-        <v>1179</v>
+        <v>171</v>
       </c>
       <c r="B652" s="1" t="s">
-        <v>1187</v>
+        <v>172</v>
       </c>
     </row>
     <row r="653" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A653" t="s">
-        <v>1195</v>
+        <v>1179</v>
       </c>
       <c r="B653" s="1" t="s">
-        <v>1203</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="654" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
-        <v>173</v>
+        <v>1195</v>
       </c>
       <c r="B654" s="1" t="s">
-        <v>174</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="655" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B655" s="1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="656" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B656" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="657" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>600</v>
+        <v>177</v>
       </c>
       <c r="B657" s="1" t="s">
-        <v>605</v>
+        <v>178</v>
       </c>
     </row>
     <row r="658" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B658" s="1" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
     </row>
     <row r="659" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B659" s="1" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="660" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A660" t="s">
-        <v>179</v>
+        <v>602</v>
       </c>
       <c r="B660" s="1" t="s">
-        <v>180</v>
+        <v>610</v>
       </c>
     </row>
     <row r="661" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A661" t="s">
-        <v>1178</v>
+        <v>179</v>
       </c>
       <c r="B661" s="1" t="s">
-        <v>1186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="662" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1194</v>
+        <v>1178</v>
       </c>
       <c r="B662" s="1" t="s">
-        <v>1202</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="663" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A663" t="s">
-        <v>181</v>
+        <v>1194</v>
       </c>
       <c r="B663" s="1" t="s">
-        <v>182</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="664" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A664" t="s">
-        <v>1180</v>
+        <v>181</v>
       </c>
       <c r="B664" s="1" t="s">
-        <v>1188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="665" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A665" t="s">
-        <v>1196</v>
+        <v>1180</v>
       </c>
       <c r="B665" s="1" t="s">
-        <v>1204</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="666" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A666" t="s">
-        <v>671</v>
+        <v>1196</v>
       </c>
       <c r="B666" s="1" t="s">
-        <v>674</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="667" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A667" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B667" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="668" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A668" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B668" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="669" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A669" t="s">
-        <v>1080</v>
+        <v>673</v>
       </c>
       <c r="B669" s="1" t="s">
-        <v>476</v>
+        <v>676</v>
       </c>
     </row>
     <row r="670" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A670" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="B670" s="1" t="s">
-        <v>1064</v>
+        <v>476</v>
       </c>
     </row>
     <row r="671" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A671" t="s">
-        <v>1520</v>
+        <v>1081</v>
       </c>
       <c r="B671" s="1" t="s">
-        <v>1522</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="672" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A672" t="s">
-        <v>566</v>
+        <v>1520</v>
       </c>
       <c r="B672" s="1" t="s">
-        <v>568</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="673" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A673" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B673" s="1" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="674" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A674" t="s">
-        <v>1518</v>
+        <v>567</v>
       </c>
       <c r="B674" s="1" t="s">
-        <v>1521</v>
+        <v>569</v>
       </c>
     </row>
     <row r="675" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A675" t="s">
-        <v>1027</v>
+        <v>1518</v>
       </c>
       <c r="B675" s="1" t="s">
-        <v>1035</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="676" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A676" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B676" s="1" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="677" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A677" t="s">
-        <v>947</v>
+        <v>1028</v>
       </c>
       <c r="B677" s="1" t="s">
-        <v>948</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="678" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A678" t="s">
-        <v>923</v>
+        <v>947</v>
       </c>
       <c r="B678" s="1" t="s">
-        <v>926</v>
+        <v>948</v>
       </c>
     </row>
     <row r="679" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A679" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B679" s="1" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="680" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A680" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="B680" s="1" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="681" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A681" t="s">
-        <v>908</v>
+        <v>925</v>
       </c>
       <c r="B681" s="1" t="s">
-        <v>912</v>
+        <v>928</v>
       </c>
     </row>
     <row r="682" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A682" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="B682" s="1" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
     </row>
     <row r="683" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A683" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="B683" s="1" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
     </row>
     <row r="684" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A684" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="B684" s="1" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
     </row>
     <row r="685" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A685" t="s">
-        <v>574</v>
+        <v>911</v>
       </c>
       <c r="B685" s="1" t="s">
-        <v>575</v>
+        <v>915</v>
       </c>
     </row>
     <row r="686" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A686" t="s">
-        <v>629</v>
+        <v>574</v>
       </c>
       <c r="B686" s="1" t="s">
-        <v>631</v>
+        <v>575</v>
       </c>
     </row>
     <row r="687" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A687" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B687" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="688" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A688" t="s">
-        <v>1308</v>
+        <v>630</v>
       </c>
       <c r="B688" s="1" t="s">
-        <v>1310</v>
+        <v>632</v>
       </c>
     </row>
     <row r="689" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A689" t="s">
-        <v>866</v>
+        <v>1308</v>
       </c>
       <c r="B689" s="1" t="s">
-        <v>862</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="690" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A690" t="s">
-        <v>877</v>
+        <v>866</v>
       </c>
       <c r="B690" s="1" t="s">
-        <v>880</v>
+        <v>862</v>
       </c>
     </row>
     <row r="691" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A691" t="s">
-        <v>884</v>
+        <v>877</v>
       </c>
       <c r="B691" s="1" t="s">
-        <v>887</v>
+        <v>880</v>
       </c>
     </row>
     <row r="692" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A692" t="s">
-        <v>865</v>
+        <v>884</v>
       </c>
       <c r="B692" s="1" t="s">
-        <v>861</v>
+        <v>887</v>
       </c>
     </row>
     <row r="693" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A693" t="s">
-        <v>878</v>
+        <v>865</v>
       </c>
       <c r="B693" s="1" t="s">
-        <v>881</v>
+        <v>861</v>
       </c>
     </row>
     <row r="694" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A694" t="s">
-        <v>885</v>
+        <v>878</v>
       </c>
       <c r="B694" s="1" t="s">
-        <v>888</v>
+        <v>881</v>
       </c>
     </row>
     <row r="695" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A695" t="s">
-        <v>899</v>
+        <v>885</v>
       </c>
       <c r="B695" s="1" t="s">
-        <v>864</v>
+        <v>888</v>
       </c>
     </row>
     <row r="696" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A696" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="B696" s="1" t="s">
-        <v>882</v>
+        <v>864</v>
       </c>
     </row>
     <row r="697" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A697" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="B697" s="1" t="s">
-        <v>889</v>
+        <v>882</v>
       </c>
     </row>
     <row r="698" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A698" t="s">
-        <v>867</v>
+        <v>901</v>
       </c>
       <c r="B698" s="1" t="s">
-        <v>863</v>
+        <v>889</v>
       </c>
     </row>
     <row r="699" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A699" t="s">
-        <v>879</v>
+        <v>867</v>
       </c>
       <c r="B699" s="1" t="s">
-        <v>883</v>
+        <v>863</v>
       </c>
     </row>
     <row r="700" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A700" t="s">
-        <v>886</v>
+        <v>879</v>
       </c>
       <c r="B700" s="1" t="s">
-        <v>890</v>
+        <v>883</v>
       </c>
     </row>
     <row r="701" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A701" t="s">
-        <v>1210</v>
+        <v>886</v>
       </c>
       <c r="B701" s="1" t="s">
-        <v>1216</v>
+        <v>890</v>
       </c>
     </row>
     <row r="702" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A702" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="B702" s="1" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="703" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A703" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="B703" s="1" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="704" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A704" t="s">
-        <v>1456</v>
+        <v>1212</v>
       </c>
       <c r="B704" s="1" t="s">
-        <v>1457</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="705" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A705" t="s">
-        <v>1464</v>
+        <v>1456</v>
       </c>
       <c r="B705" s="1" t="s">
-        <v>1466</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="706" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A706" t="s">
-        <v>1459</v>
+        <v>1464</v>
       </c>
       <c r="B706" s="1" t="s">
-        <v>1462</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="707" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A707" t="s">
-        <v>1465</v>
+        <v>1459</v>
       </c>
       <c r="B707" s="1" t="s">
-        <v>1467</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="708" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A708" t="s">
-        <v>786</v>
+        <v>1465</v>
       </c>
       <c r="B708" s="1" t="s">
-        <v>442</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="709" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A709" t="s">
-        <v>996</v>
+        <v>786</v>
       </c>
       <c r="B709" s="1" t="s">
-        <v>974</v>
+        <v>442</v>
       </c>
     </row>
     <row r="710" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A710" t="s">
-        <v>1066</v>
+        <v>996</v>
       </c>
       <c r="B710" s="1" t="s">
-        <v>1065</v>
+        <v>974</v>
       </c>
     </row>
     <row r="711" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A711" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B711" s="1" t="s">
-        <v>1070</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="712" spans="1:2" x14ac:dyDescent="0.35">
@@ -11842,415 +11848,415 @@
         <v>1067</v>
       </c>
       <c r="B712" s="1" t="s">
-        <v>1516</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="713" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A713" t="s">
-        <v>778</v>
+        <v>1067</v>
       </c>
       <c r="B713" s="1" t="s">
-        <v>780</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="714" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A714" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="B714" s="1" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="715" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A715" t="s">
-        <v>682</v>
+        <v>779</v>
       </c>
       <c r="B715" s="1" t="s">
-        <v>685</v>
+        <v>781</v>
       </c>
     </row>
     <row r="716" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A716" t="s">
-        <v>183</v>
+        <v>682</v>
       </c>
       <c r="B716" s="1" t="s">
-        <v>184</v>
+        <v>685</v>
       </c>
     </row>
     <row r="717" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A717" t="s">
-        <v>1312</v>
+        <v>183</v>
       </c>
       <c r="B717" s="1" t="s">
-        <v>1320</v>
+        <v>184</v>
       </c>
     </row>
     <row r="718" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A718" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="B718" s="1" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="719" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A719" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="B719" s="1" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="720" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A720" t="s">
-        <v>1661</v>
+        <v>1314</v>
       </c>
       <c r="B720" s="1" t="s">
-        <v>1683</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="721" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A721" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="B721" s="1" t="s">
-        <v>1684</v>
+        <v>1683</v>
       </c>
     </row>
     <row r="722" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A722" t="s">
-        <v>1669</v>
+        <v>1662</v>
       </c>
       <c r="B722" s="1" t="s">
-        <v>1687</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="723" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A723" t="s">
-        <v>1670</v>
+        <v>1669</v>
       </c>
       <c r="B723" s="1" t="s">
-        <v>1691</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="724" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A724" t="s">
-        <v>185</v>
+        <v>1670</v>
       </c>
       <c r="B724" s="1" t="s">
-        <v>186</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="725" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A725" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B725" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="726" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A726" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B726" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="727" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A727" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B727" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="728" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A728" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B728" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="729" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A729" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B729" s="1" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
     </row>
     <row r="730" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A730" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B730" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="731" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A731" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B731" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="732" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A732" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B732" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="733" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A733" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B733" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="734" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A734" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B734" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="735" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A735" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B735" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="736" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A736" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B736" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="737" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A737" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B737" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="738" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A738" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B738" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="739" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A739" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B739" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="740" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A740" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B740" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="741" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A741" t="s">
-        <v>742</v>
+        <v>206</v>
       </c>
       <c r="B741" s="1" t="s">
-        <v>812</v>
+        <v>164</v>
       </c>
     </row>
     <row r="742" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A742" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="B742" s="1" t="s">
-        <v>718</v>
+        <v>812</v>
       </c>
     </row>
     <row r="743" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A743" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B743" s="1" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="744" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A744" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B744" s="1" t="s">
-        <v>813</v>
+        <v>719</v>
       </c>
     </row>
     <row r="745" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A745" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B745" s="1" t="s">
-        <v>706</v>
+        <v>813</v>
       </c>
     </row>
     <row r="746" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A746" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B746" s="1" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="747" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A747" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="B747" s="1" t="s">
-        <v>814</v>
+        <v>707</v>
       </c>
     </row>
     <row r="748" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A748" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B748" s="1" t="s">
-        <v>712</v>
+        <v>814</v>
       </c>
     </row>
     <row r="749" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A749" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B749" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="750" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A750" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B750" s="1" t="s">
-        <v>815</v>
+        <v>713</v>
       </c>
     </row>
     <row r="751" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A751" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B751" s="1" t="s">
-        <v>709</v>
+        <v>815</v>
       </c>
     </row>
     <row r="752" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A752" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B752" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="753" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A753" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B753" s="1" t="s">
-        <v>816</v>
+        <v>710</v>
       </c>
     </row>
     <row r="754" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A754" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B754" s="1" t="s">
-        <v>721</v>
+        <v>816</v>
       </c>
     </row>
     <row r="755" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A755" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B755" s="1" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="756" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A756" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B756" s="1" t="s">
-        <v>817</v>
+        <v>722</v>
       </c>
     </row>
     <row r="757" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A757" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="B757" s="1" t="s">
-        <v>715</v>
+        <v>817</v>
       </c>
     </row>
     <row r="758" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A758" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="B758" s="1" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="759" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A759" t="s">
-        <v>1250</v>
+        <v>759</v>
       </c>
       <c r="B759" s="1" t="s">
-        <v>1245</v>
+        <v>716</v>
       </c>
     </row>
     <row r="760" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A760" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="B760" s="1" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="761" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A761" t="s">
-        <v>1254</v>
+        <v>1251</v>
       </c>
       <c r="B761" s="1" t="s">
-        <v>1255</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="762" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A762" t="s">
-        <v>1494</v>
+        <v>1254</v>
       </c>
       <c r="B762" s="1" t="s">
-        <v>1496</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="763" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A763" t="s">
-        <v>1498</v>
+        <v>1494</v>
       </c>
       <c r="B763" s="1" t="s">
-        <v>1505</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="764" spans="1:3" x14ac:dyDescent="0.35">
@@ -12258,509 +12264,509 @@
         <v>1498</v>
       </c>
       <c r="B764" s="1" t="s">
-        <v>1503</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="765" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A765" t="s">
-        <v>1499</v>
+        <v>1498</v>
       </c>
       <c r="B765" s="1" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="766" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A766" t="s">
-        <v>1552</v>
+        <v>1499</v>
       </c>
       <c r="B766" s="1" t="s">
-        <v>1542</v>
-      </c>
-      <c r="C766" s="2" t="s">
-        <v>1546</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="767" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A767" t="s">
-        <v>1553</v>
+        <v>1552</v>
       </c>
       <c r="B767" s="1" t="s">
-        <v>1543</v>
+        <v>1542</v>
       </c>
       <c r="C767" s="2" t="s">
-        <v>1547</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="768" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A768" t="s">
-        <v>1714</v>
+        <v>1553</v>
       </c>
       <c r="B768" s="1" t="s">
-        <v>1724</v>
+        <v>1543</v>
+      </c>
+      <c r="C768" s="2" t="s">
+        <v>1547</v>
       </c>
     </row>
     <row r="769" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A769" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="B769" s="1" t="s">
-        <v>1726</v>
+        <v>1724</v>
       </c>
     </row>
     <row r="770" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A770" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="B770" s="1" t="s">
-        <v>1725</v>
+        <v>1726</v>
       </c>
     </row>
     <row r="771" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A771" t="s">
-        <v>1057</v>
+        <v>1716</v>
       </c>
       <c r="B771" s="1" t="s">
-        <v>1061</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="772" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A772" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B772" s="1" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="773" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A773" t="s">
-        <v>1529</v>
+        <v>1058</v>
       </c>
       <c r="B773" s="1" t="s">
-        <v>1530</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="774" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A774" t="s">
-        <v>339</v>
+        <v>1529</v>
       </c>
       <c r="B774" s="1" t="s">
-        <v>341</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="775" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A775" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="B775" s="1" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="776" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A776" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B776" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="777" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A777" t="s">
-        <v>1226</v>
+        <v>347</v>
       </c>
       <c r="B777" s="1" t="s">
-        <v>1232</v>
+        <v>343</v>
       </c>
     </row>
     <row r="778" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A778" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="B778" s="1" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="779" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A779" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="B779" s="1" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="780" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A780" t="s">
-        <v>921</v>
+        <v>1228</v>
       </c>
       <c r="B780" s="1" t="s">
-        <v>919</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="781" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A781" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="B781" s="1" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
     </row>
     <row r="782" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A782" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="B782" s="1" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
     </row>
     <row r="783" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A783" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="B783" s="1" t="s">
-        <v>939</v>
+        <v>922</v>
       </c>
     </row>
     <row r="784" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A784" t="s">
-        <v>940</v>
+        <v>918</v>
       </c>
       <c r="B784" s="1" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
     </row>
     <row r="785" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A785" t="s">
-        <v>558</v>
+        <v>940</v>
       </c>
       <c r="B785" s="1" t="s">
-        <v>559</v>
+        <v>941</v>
       </c>
     </row>
     <row r="786" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A786" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B786" s="1" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
     <row r="787" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A787" t="s">
-        <v>1332</v>
+        <v>560</v>
       </c>
       <c r="B787" s="1" t="s">
-        <v>1338</v>
+        <v>561</v>
       </c>
     </row>
     <row r="788" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A788" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B788" s="1" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="789" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A789" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B789" s="1" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="790" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A790" t="s">
-        <v>584</v>
+        <v>1334</v>
       </c>
       <c r="B790" s="1" t="s">
-        <v>587</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="791" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A791" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="B791" s="1" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
     </row>
     <row r="792" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A792" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B792" s="1" t="s">
-        <v>595</v>
+        <v>590</v>
       </c>
     </row>
     <row r="793" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A793" t="s">
-        <v>371</v>
+        <v>589</v>
       </c>
       <c r="B793" s="1" t="s">
-        <v>377</v>
+        <v>595</v>
       </c>
     </row>
     <row r="794" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A794" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B794" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="795" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A795" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B795" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="796" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A796" t="s">
-        <v>681</v>
+        <v>375</v>
       </c>
       <c r="B796" s="1" t="s">
-        <v>618</v>
+        <v>379</v>
       </c>
     </row>
     <row r="797" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A797" t="s">
-        <v>351</v>
+        <v>681</v>
       </c>
       <c r="B797" s="1" t="s">
-        <v>352</v>
+        <v>618</v>
       </c>
     </row>
     <row r="798" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A798" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="B798" s="1" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="799" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A799" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B799" s="1" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="800" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A800" t="s">
-        <v>1297</v>
+        <v>360</v>
       </c>
       <c r="B800" s="1" t="s">
-        <v>1300</v>
+        <v>356</v>
       </c>
     </row>
     <row r="801" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A801" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="B801" s="1" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="802" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A802" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="B802" s="1" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="803" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A803" t="s">
-        <v>1509</v>
+        <v>1299</v>
       </c>
       <c r="B803" s="1" t="s">
-        <v>1511</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="804" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A804" t="s">
-        <v>1705</v>
+        <v>1509</v>
       </c>
       <c r="B804" s="1" t="s">
-        <v>1712</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="805" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A805" t="s">
-        <v>1703</v>
+        <v>1705</v>
       </c>
       <c r="B805" s="1" t="s">
-        <v>1710</v>
+        <v>1712</v>
       </c>
     </row>
     <row r="806" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A806" t="s">
-        <v>1704</v>
+        <v>1703</v>
       </c>
       <c r="B806" s="1" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="807" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A807" t="s">
-        <v>997</v>
+        <v>1704</v>
       </c>
       <c r="B807" s="1" t="s">
-        <v>961</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="808" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A808" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B808" s="1" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="809" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A809" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B809" s="1" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="810" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A810" t="s">
-        <v>1627</v>
+        <v>999</v>
       </c>
       <c r="B810" s="1" t="s">
-        <v>1636</v>
+        <v>963</v>
       </c>
     </row>
     <row r="811" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A811" t="s">
-        <v>1628</v>
+        <v>1627</v>
       </c>
       <c r="B811" s="1" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="812" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A812" t="s">
-        <v>853</v>
+        <v>1628</v>
       </c>
       <c r="B812" s="1" t="s">
-        <v>854</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="813" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A813" t="s">
-        <v>851</v>
+        <v>853</v>
       </c>
       <c r="B813" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="814" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A814" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B814" s="1" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="815" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A815" t="s">
-        <v>776</v>
+        <v>852</v>
       </c>
       <c r="B815" s="1" t="s">
-        <v>774</v>
+        <v>856</v>
       </c>
     </row>
     <row r="816" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A816" t="s">
-        <v>207</v>
+        <v>776</v>
       </c>
       <c r="B816" s="1" t="s">
-        <v>208</v>
+        <v>774</v>
       </c>
     </row>
     <row r="817" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A817" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B817" s="1" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="818" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A818" t="s">
-        <v>701</v>
+        <v>209</v>
       </c>
       <c r="B818" s="1" t="s">
-        <v>664</v>
+        <v>210</v>
       </c>
     </row>
     <row r="819" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A819" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B819" s="1" t="s">
-        <v>540</v>
+        <v>664</v>
       </c>
     </row>
     <row r="820" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A820" t="s">
-        <v>760</v>
+        <v>702</v>
       </c>
       <c r="B820" s="1" t="s">
-        <v>523</v>
+        <v>540</v>
       </c>
     </row>
     <row r="821" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A821" t="s">
-        <v>1348</v>
+        <v>760</v>
       </c>
       <c r="B821" s="1" t="s">
-        <v>1349</v>
+        <v>523</v>
       </c>
     </row>
     <row r="822" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A822" t="s">
-        <v>703</v>
+        <v>1348</v>
       </c>
       <c r="B822" s="1" t="s">
-        <v>524</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="823" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A823" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B823" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="824" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A824" t="s">
-        <v>761</v>
+        <v>704</v>
       </c>
       <c r="B824" s="1" t="s">
-        <v>763</v>
+        <v>525</v>
       </c>
     </row>
     <row r="825" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A825" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B825" s="1" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="826" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A826" t="s">
-        <v>1694</v>
+        <v>762</v>
       </c>
       <c r="B826" s="1" t="s">
-        <v>1699</v>
+        <v>764</v>
       </c>
     </row>
     <row r="827" spans="1:2" x14ac:dyDescent="0.35">
@@ -12768,15 +12774,15 @@
         <v>1694</v>
       </c>
       <c r="B827" s="1" t="s">
-        <v>1692</v>
+        <v>1699</v>
       </c>
     </row>
     <row r="828" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A828" t="s">
-        <v>1695</v>
+        <v>1694</v>
       </c>
       <c r="B828" s="1" t="s">
-        <v>1698</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="829" spans="1:2" x14ac:dyDescent="0.35">
@@ -12784,840 +12790,848 @@
         <v>1695</v>
       </c>
       <c r="B829" s="1" t="s">
-        <v>1700</v>
+        <v>1698</v>
       </c>
     </row>
     <row r="830" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A830" t="s">
-        <v>1655</v>
+        <v>1695</v>
       </c>
       <c r="B830" s="1" t="s">
-        <v>1677</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="831" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A831" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="B831" s="1" t="s">
-        <v>1680</v>
+        <v>1677</v>
       </c>
     </row>
     <row r="832" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A832" t="s">
-        <v>1653</v>
+        <v>1656</v>
       </c>
       <c r="B832" s="1" t="s">
-        <v>1678</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="833" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A833" t="s">
-        <v>1654</v>
+        <v>1653</v>
       </c>
       <c r="B833" s="1" t="s">
-        <v>1679</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="834" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A834" t="s">
-        <v>1352</v>
+        <v>1654</v>
       </c>
       <c r="B834" s="1" t="s">
-        <v>1360</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="835" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A835" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="B835" s="1" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="836" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A836" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="B836" s="1" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="837" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A837" t="s">
-        <v>693</v>
+        <v>1354</v>
       </c>
       <c r="B837" s="1" t="s">
-        <v>692</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="838" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A838" t="s">
-        <v>906</v>
+        <v>693</v>
       </c>
       <c r="B838" s="1" t="s">
-        <v>665</v>
+        <v>692</v>
       </c>
     </row>
     <row r="839" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A839" t="s">
-        <v>819</v>
+        <v>906</v>
       </c>
       <c r="B839" s="1" t="s">
-        <v>810</v>
+        <v>665</v>
       </c>
     </row>
     <row r="840" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A840" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="B840" s="1" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
     </row>
     <row r="841" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A841" t="s">
-        <v>1606</v>
+        <v>818</v>
       </c>
       <c r="B841" s="1" t="s">
-        <v>1617</v>
+        <v>811</v>
       </c>
     </row>
     <row r="842" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A842" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="B842" s="1" t="s">
-        <v>1621</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="843" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A843" t="s">
-        <v>1570</v>
+        <v>1605</v>
       </c>
       <c r="B843" s="1" t="s">
-        <v>1566</v>
+        <v>1621</v>
       </c>
     </row>
     <row r="844" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A844" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="B844" s="1" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="845" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A845" t="s">
-        <v>1567</v>
+        <v>1569</v>
       </c>
       <c r="B845" s="1" t="s">
-        <v>1563</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="846" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A846" t="s">
-        <v>1568</v>
+        <v>1567</v>
       </c>
       <c r="B846" s="1" t="s">
-        <v>1564</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="847" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A847" t="s">
-        <v>1608</v>
+        <v>1568</v>
       </c>
       <c r="B847" s="1" t="s">
-        <v>1618</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="848" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A848" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="B848" s="1" t="s">
-        <v>1622</v>
+        <v>1618</v>
       </c>
     </row>
     <row r="849" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A849" t="s">
-        <v>1371</v>
+        <v>1607</v>
       </c>
       <c r="B849" s="1" t="s">
-        <v>1369</v>
+        <v>1622</v>
       </c>
     </row>
     <row r="850" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A850" t="s">
-        <v>492</v>
+        <v>1371</v>
       </c>
       <c r="B850" s="1" t="s">
-        <v>494</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="851" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A851" t="s">
-        <v>823</v>
+        <v>492</v>
       </c>
       <c r="B851" s="1" t="s">
-        <v>828</v>
+        <v>494</v>
       </c>
     </row>
     <row r="852" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A852" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B852" s="1" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
     </row>
     <row r="853" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A853" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B853" s="1" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
     </row>
     <row r="854" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A854" t="s">
-        <v>668</v>
+        <v>825</v>
       </c>
       <c r="B854" s="1" t="s">
-        <v>658</v>
+        <v>826</v>
       </c>
     </row>
     <row r="855" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A855" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="B855" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="856" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A856" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B856" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="857" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A857" t="s">
-        <v>1376</v>
+        <v>667</v>
       </c>
       <c r="B857" s="1" t="s">
-        <v>1374</v>
+        <v>660</v>
       </c>
     </row>
     <row r="858" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A858" t="s">
-        <v>1373</v>
+        <v>1376</v>
       </c>
       <c r="B858" s="1" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="859" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A859" t="s">
-        <v>1377</v>
+        <v>1373</v>
       </c>
       <c r="B859" s="1" t="s">
-        <v>1379</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="860" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A860" t="s">
-        <v>1378</v>
+        <v>1377</v>
       </c>
       <c r="B860" s="1" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="861" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A861" t="s">
-        <v>977</v>
+        <v>1378</v>
       </c>
       <c r="B861" s="1" t="s">
-        <v>979</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="862" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A862" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B862" s="1" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="863" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A863" t="s">
-        <v>362</v>
+        <v>978</v>
       </c>
       <c r="B863" s="1" t="s">
-        <v>363</v>
+        <v>980</v>
       </c>
     </row>
     <row r="864" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A864" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="B864" s="1" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="865" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A865" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B865" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="866" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A866" t="s">
-        <v>1050</v>
+        <v>368</v>
       </c>
       <c r="B866" s="1" t="s">
-        <v>1051</v>
-      </c>
-      <c r="C866" s="2" t="s">
-        <v>1052</v>
+        <v>366</v>
       </c>
     </row>
     <row r="867" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A867" t="s">
-        <v>211</v>
+        <v>1050</v>
       </c>
       <c r="B867" s="1" t="s">
-        <v>212</v>
+        <v>1051</v>
       </c>
       <c r="C867" s="2" t="s">
-        <v>212</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="868" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A868" t="s">
-        <v>299</v>
+        <v>211</v>
       </c>
       <c r="B868" s="1" t="s">
-        <v>301</v>
+        <v>212</v>
       </c>
       <c r="C868" s="2" t="s">
-        <v>300</v>
+        <v>212</v>
       </c>
     </row>
     <row r="869" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A869" t="s">
-        <v>213</v>
+        <v>299</v>
       </c>
       <c r="B869" s="1" t="s">
-        <v>214</v>
+        <v>301</v>
       </c>
       <c r="C869" s="2" t="s">
-        <v>251</v>
+        <v>300</v>
       </c>
     </row>
     <row r="870" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A870" t="s">
-        <v>439</v>
+        <v>213</v>
       </c>
       <c r="B870" s="1" t="s">
-        <v>447</v>
+        <v>214</v>
+      </c>
+      <c r="C870" s="2" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="871" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A871" t="s">
-        <v>1055</v>
+        <v>439</v>
       </c>
       <c r="B871" s="1" t="s">
-        <v>1047</v>
-      </c>
-      <c r="C871" s="2" t="s">
-        <v>1048</v>
+        <v>447</v>
       </c>
     </row>
     <row r="872" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A872" t="s">
-        <v>215</v>
+        <v>1055</v>
       </c>
       <c r="B872" s="1" t="s">
-        <v>579</v>
+        <v>1047</v>
       </c>
       <c r="C872" s="2" t="s">
-        <v>580</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="873" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A873" t="s">
-        <v>260</v>
+        <v>215</v>
       </c>
       <c r="B873" s="1" t="s">
-        <v>265</v>
+        <v>579</v>
       </c>
       <c r="C873" s="2" t="s">
-        <v>262</v>
+        <v>580</v>
       </c>
     </row>
     <row r="874" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A874" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B874" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C874" s="2" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
     </row>
     <row r="875" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A875" t="s">
-        <v>216</v>
+        <v>261</v>
       </c>
       <c r="B875" s="1" t="s">
-        <v>217</v>
+        <v>264</v>
       </c>
       <c r="C875" s="2" t="s">
-        <v>217</v>
+        <v>268</v>
       </c>
     </row>
     <row r="876" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A876" t="s">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="B876" s="1" t="s">
-        <v>247</v>
+        <v>217</v>
       </c>
       <c r="C876" s="2" t="s">
-        <v>250</v>
+        <v>217</v>
       </c>
     </row>
     <row r="877" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A877" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B877" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C877" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="878" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A878" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
       <c r="B878" s="1" t="s">
-        <v>219</v>
+        <v>246</v>
       </c>
       <c r="C878" s="2" t="s">
-        <v>219</v>
+        <v>249</v>
       </c>
     </row>
     <row r="879" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A879" t="s">
-        <v>987</v>
+        <v>218</v>
       </c>
       <c r="B879" s="1" t="s">
-        <v>995</v>
+        <v>219</v>
+      </c>
+      <c r="C879" s="2" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="880" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A880" t="s">
-        <v>1732</v>
+        <v>987</v>
       </c>
       <c r="B880" s="1" t="s">
-        <v>1731</v>
+        <v>995</v>
       </c>
     </row>
     <row r="881" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A881" t="s">
-        <v>1671</v>
+        <v>1732</v>
       </c>
       <c r="B881" s="1" t="s">
-        <v>1672</v>
+        <v>1731</v>
       </c>
     </row>
     <row r="882" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A882" t="s">
-        <v>1729</v>
+        <v>1671</v>
       </c>
       <c r="B882" s="1" t="s">
-        <v>1730</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="883" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A883" t="s">
-        <v>281</v>
+        <v>1729</v>
       </c>
       <c r="B883" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="C883" s="2" t="s">
-        <v>283</v>
+        <v>1730</v>
       </c>
     </row>
     <row r="884" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A884" t="s">
-        <v>986</v>
+        <v>281</v>
       </c>
       <c r="B884" s="1" t="s">
-        <v>994</v>
+        <v>282</v>
+      </c>
+      <c r="C884" s="2" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="885" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A885" t="s">
-        <v>799</v>
+        <v>986</v>
       </c>
       <c r="B885" s="1" t="s">
-        <v>802</v>
+        <v>994</v>
       </c>
     </row>
     <row r="886" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A886" t="s">
-        <v>258</v>
+        <v>799</v>
       </c>
       <c r="B886" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="C886" s="2" t="s">
-        <v>263</v>
+        <v>802</v>
       </c>
     </row>
     <row r="887" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A887" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B887" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C887" s="2" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
     </row>
     <row r="888" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A888" t="s">
-        <v>297</v>
+        <v>259</v>
       </c>
       <c r="B888" s="1" t="s">
-        <v>303</v>
+        <v>267</v>
       </c>
       <c r="C888" s="2" t="s">
-        <v>307</v>
+        <v>269</v>
       </c>
     </row>
     <row r="889" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A889" t="s">
-        <v>220</v>
+        <v>297</v>
       </c>
       <c r="B889" s="1" t="s">
-        <v>1257</v>
+        <v>303</v>
       </c>
       <c r="C889" s="2" t="s">
-        <v>221</v>
+        <v>307</v>
       </c>
     </row>
     <row r="890" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A890" t="s">
-        <v>988</v>
+        <v>220</v>
       </c>
       <c r="B890" s="1" t="s">
-        <v>1258</v>
+        <v>1257</v>
+      </c>
+      <c r="C890" s="2" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="891" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A891" t="s">
-        <v>1733</v>
+        <v>988</v>
       </c>
       <c r="B891" s="1" t="s">
-        <v>1734</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="892" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A892" t="s">
-        <v>298</v>
+        <v>1733</v>
       </c>
       <c r="B892" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="C892" s="2" t="s">
-        <v>308</v>
+        <v>1734</v>
       </c>
     </row>
     <row r="893" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A893" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="B893" s="1" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C893" s="2" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
     </row>
     <row r="894" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A894" t="s">
-        <v>222</v>
+        <v>294</v>
       </c>
       <c r="B894" s="1" t="s">
-        <v>223</v>
+        <v>306</v>
       </c>
       <c r="C894" s="2" t="s">
-        <v>257</v>
+        <v>314</v>
       </c>
     </row>
     <row r="895" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A895" t="s">
-        <v>985</v>
+        <v>222</v>
       </c>
       <c r="B895" s="1" t="s">
-        <v>993</v>
+        <v>223</v>
+      </c>
+      <c r="C895" s="2" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="896" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A896" t="s">
-        <v>800</v>
+        <v>985</v>
       </c>
       <c r="B896" s="1" t="s">
-        <v>805</v>
+        <v>993</v>
       </c>
     </row>
     <row r="897" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A897" t="s">
-        <v>224</v>
+        <v>800</v>
       </c>
       <c r="B897" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="C897" s="2" t="s">
-        <v>225</v>
+        <v>805</v>
       </c>
     </row>
     <row r="898" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A898" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="B898" s="1" t="s">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="C898" s="2" t="s">
-        <v>248</v>
+        <v>225</v>
       </c>
     </row>
     <row r="899" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A899" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B899" s="1" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C899" s="2" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="900" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A900" t="s">
-        <v>562</v>
+        <v>239</v>
       </c>
       <c r="B900" s="1" t="s">
-        <v>563</v>
+        <v>245</v>
+      </c>
+      <c r="C900" s="2" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="901" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A901" t="s">
-        <v>989</v>
+        <v>562</v>
       </c>
       <c r="B901" s="1" t="s">
-        <v>992</v>
+        <v>563</v>
       </c>
     </row>
     <row r="902" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A902" t="s">
-        <v>564</v>
+        <v>989</v>
       </c>
       <c r="B902" s="1" t="s">
-        <v>565</v>
+        <v>992</v>
       </c>
     </row>
     <row r="903" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A903" t="s">
-        <v>797</v>
+        <v>564</v>
       </c>
       <c r="B903" s="1" t="s">
-        <v>803</v>
+        <v>565</v>
       </c>
     </row>
     <row r="904" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A904" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B904" s="1" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="905" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A905" t="s">
-        <v>330</v>
+        <v>798</v>
       </c>
       <c r="B905" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="C905" s="2" t="s">
-        <v>336</v>
+        <v>804</v>
       </c>
     </row>
     <row r="906" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A906" t="s">
-        <v>983</v>
+        <v>330</v>
       </c>
       <c r="B906" s="1" t="s">
-        <v>990</v>
+        <v>335</v>
+      </c>
+      <c r="C906" s="2" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="907" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A907" t="s">
-        <v>1735</v>
+        <v>983</v>
       </c>
       <c r="B907" s="1" t="s">
-        <v>1736</v>
+        <v>990</v>
       </c>
     </row>
     <row r="908" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A908" t="s">
-        <v>801</v>
+        <v>1735</v>
       </c>
       <c r="B908" s="1" t="s">
-        <v>806</v>
+        <v>1736</v>
       </c>
     </row>
     <row r="909" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A909" t="s">
-        <v>296</v>
+        <v>801</v>
       </c>
       <c r="B909" s="1" t="s">
-        <v>302</v>
+        <v>806</v>
       </c>
     </row>
     <row r="910" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A910" t="s">
-        <v>226</v>
+        <v>296</v>
       </c>
       <c r="B910" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="C910" s="2" t="s">
-        <v>292</v>
+        <v>302</v>
       </c>
     </row>
     <row r="911" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A911" t="s">
-        <v>984</v>
+        <v>226</v>
       </c>
       <c r="B911" s="1" t="s">
-        <v>991</v>
+        <v>227</v>
+      </c>
+      <c r="C911" s="2" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="912" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A912" t="s">
-        <v>1727</v>
+        <v>984</v>
       </c>
       <c r="B912" s="1" t="s">
-        <v>1728</v>
+        <v>991</v>
       </c>
     </row>
     <row r="913" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A913" t="s">
-        <v>228</v>
+        <v>1727</v>
       </c>
       <c r="B913" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="C913" s="2" t="s">
-        <v>229</v>
+        <v>1728</v>
       </c>
     </row>
     <row r="914" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A914" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B914" s="1" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="C914" s="2" t="s">
-        <v>253</v>
+        <v>229</v>
       </c>
     </row>
     <row r="915" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A915" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B915" s="1" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C915" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="916" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A916" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="B916" s="1" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="C916" s="2" t="s">
-        <v>231</v>
+        <v>254</v>
       </c>
     </row>
     <row r="917" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A917" t="s">
-        <v>1046</v>
+        <v>230</v>
       </c>
       <c r="B917" s="1" t="s">
-        <v>1049</v>
+        <v>231</v>
       </c>
       <c r="C917" s="2" t="s">
-        <v>1053</v>
+        <v>231</v>
       </c>
     </row>
     <row r="918" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A918" t="s">
-        <v>233</v>
+        <v>1046</v>
       </c>
       <c r="B918" s="1" t="s">
-        <v>242</v>
+        <v>1049</v>
       </c>
       <c r="C918" s="2" t="s">
-        <v>255</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="919" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A919" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B919" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C919" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="920" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A920" t="s">
+        <v>237</v>
+      </c>
+      <c r="B920" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C920" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="921" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A921" t="s">
         <v>295</v>
       </c>
-      <c r="B920" s="1" t="s">
+      <c r="B921" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="C920" s="2" t="s">
+      <c r="C921" s="2" t="s">
         <v>313</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K920">
-    <sortState ref="A2:K920">
-      <sortCondition ref="A1:A920"/>
+  <autoFilter ref="A1:K921">
+    <sortState ref="A2:K921">
+      <sortCondition ref="A1:A921"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
there is now a flux capacitor
</commit_message>
<xml_diff>
--- a/gui/rebalance_localizations.xlsx
+++ b/gui/rebalance_localizations.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1925" uniqueCount="1739">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1925" uniqueCount="1741">
   <si>
     <t>ENGLISH</t>
   </si>
@@ -5197,9 +5197,6 @@
     <t>Synthetic production of Morphium from a mix of heavy radioactive isotopes contained in Fissonium Flux</t>
   </si>
   <si>
-    <t>Morphium Synthethiser</t>
-  </si>
-  <si>
     <t>Optimized Morphium Synthethiser</t>
   </si>
   <si>
@@ -5240,6 +5237,15 @@
   </si>
   <si>
     <t>gui/menu/research/name/ammo_explosive_fissonium</t>
+  </si>
+  <si>
+    <t>Morphing Flux Capacitor</t>
+  </si>
+  <si>
+    <t>Advanced Morphing Flux Capacitor</t>
+  </si>
+  <si>
+    <t>Optimized Morphing Flux Capacitor</t>
   </si>
 </sst>
 </file>
@@ -8284,7 +8290,7 @@
         <v>1722</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>1724</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.35">
@@ -10352,7 +10358,7 @@
         <v>1718</v>
       </c>
       <c r="B525" s="1" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="526" spans="1:2" x14ac:dyDescent="0.35">
@@ -10360,7 +10366,7 @@
         <v>1719</v>
       </c>
       <c r="B526" s="1" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
     </row>
     <row r="527" spans="1:2" x14ac:dyDescent="0.35">
@@ -11125,10 +11131,10 @@
     </row>
     <row r="622" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A622" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="B622" s="1" t="s">
-        <v>1737</v>
+        <v>1736</v>
       </c>
     </row>
     <row r="623" spans="1:2" x14ac:dyDescent="0.35">
@@ -12310,7 +12316,7 @@
         <v>1714</v>
       </c>
       <c r="B769" s="1" t="s">
-        <v>1724</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="770" spans="1:2" x14ac:dyDescent="0.35">
@@ -12318,7 +12324,7 @@
         <v>1715</v>
       </c>
       <c r="B770" s="1" t="s">
-        <v>1726</v>
+        <v>1739</v>
       </c>
     </row>
     <row r="771" spans="1:2" x14ac:dyDescent="0.35">
@@ -12326,7 +12332,7 @@
         <v>1716</v>
       </c>
       <c r="B771" s="1" t="s">
-        <v>1725</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="772" spans="1:2" x14ac:dyDescent="0.35">
@@ -13239,10 +13245,10 @@
     </row>
     <row r="881" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A881" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="B881" s="1" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
     </row>
     <row r="882" spans="1:3" x14ac:dyDescent="0.35">
@@ -13255,10 +13261,10 @@
     </row>
     <row r="883" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A883" t="s">
+        <v>1728</v>
+      </c>
+      <c r="B883" s="1" t="s">
         <v>1729</v>
-      </c>
-      <c r="B883" s="1" t="s">
-        <v>1730</v>
       </c>
     </row>
     <row r="884" spans="1:3" x14ac:dyDescent="0.35">
@@ -13342,10 +13348,10 @@
     </row>
     <row r="892" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A892" t="s">
+        <v>1732</v>
+      </c>
+      <c r="B892" s="1" t="s">
         <v>1733</v>
-      </c>
-      <c r="B892" s="1" t="s">
-        <v>1734</v>
       </c>
     </row>
     <row r="893" spans="1:3" x14ac:dyDescent="0.35">
@@ -13491,10 +13497,10 @@
     </row>
     <row r="908" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A908" t="s">
+        <v>1734</v>
+      </c>
+      <c r="B908" s="1" t="s">
         <v>1735</v>
-      </c>
-      <c r="B908" s="1" t="s">
-        <v>1736</v>
       </c>
     </row>
     <row r="909" spans="1:3" x14ac:dyDescent="0.35">
@@ -13534,10 +13540,10 @@
     </row>
     <row r="913" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A913" t="s">
+        <v>1726</v>
+      </c>
+      <c r="B913" s="1" t="s">
         <v>1727</v>
-      </c>
-      <c r="B913" s="1" t="s">
-        <v>1728</v>
       </c>
     </row>
     <row r="914" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
fixing localization issues with commas
</commit_message>
<xml_diff>
--- a/gui/rebalance_localizations.xlsx
+++ b/gui/rebalance_localizations.xlsx
@@ -3320,9 +3320,6 @@
     <t>An advanced form of a wall. Instead of relying on a solid structure this version utilizes high-power laser beams to form a barrier. Coming into contact with this structure may be harmful.</t>
   </si>
   <si>
-    <t>Provides basic protection for the base. Can be built in multiple layers. Cheap, reliable and sturdy.</t>
-  </si>
-  <si>
     <t>gui/hud/building_description/wall_small_lvl_1</t>
   </si>
   <si>
@@ -3368,9 +3365,6 @@
     <t>gui/hud/building_description/wall_vine_lvl_3</t>
   </si>
   <si>
-    <t>These walls automatically recede into the ground when the Mech is close to them. This allows the user to shoot over them with ease and negates the need for building gates. Resistant to area and acid damage but very fragile to fire damage. The walls also regenerate missing hit points over time, but do not reconstruct from ruins by themselves.</t>
-  </si>
-  <si>
     <t>A defensive wall made from synthesized crystals found in the depths of the Galatean cavern network. When destroyed the wall will shatter and its shards will damage the nearby creatures.</t>
   </si>
   <si>
@@ -4748,18 +4742,6 @@
     <t>gui/menu/research/description/towers_drone_attack_lvl2_explosive</t>
   </si>
   <si>
-    <t>More advanced version of the Drone Attack Tower, with more drones which shoot rocket propelled explosives</t>
-  </si>
-  <si>
-    <t>More advanced version of the Drone Attack Tower, with more drones that shoot incindiary ammunition</t>
-  </si>
-  <si>
-    <t>More advanced version of the Drone Attack Tower, with more drones that shoot cryogenic high caliber ammunition</t>
-  </si>
-  <si>
-    <t>More advanced version of the Drone Attack Tower, with more drones that attack via lighting strikes</t>
-  </si>
-  <si>
     <t>Spawns defensive drones which hoover in the tower's operational radius and attack with cryogenic high caliber ammunition.</t>
   </si>
   <si>
@@ -5048,12 +5030,6 @@
     <t>HCM Tower (cryo)</t>
   </si>
   <si>
-    <t>A silo, housing a massive rocket launched vertically and aimed at distant targets. Once the rocket reaches destination, it releases multiple explosive devices that cover a very large area with acidic substance</t>
-  </si>
-  <si>
-    <t>A silo, housing a massive rocket launched vertically and aimed at distant targets. Once the rocket reaches destination, it releases multiple explosive devices that cover a very large area with a cryogenic shock</t>
-  </si>
-  <si>
     <t>HCM Tower Acid Warhead</t>
   </si>
   <si>
@@ -5093,9 +5069,6 @@
     <t>Enables a Nuclear Powerplant variant which is able to use raw uranium. Requres deuterium based heavy water as moderator and coolant.</t>
   </si>
   <si>
-    <t>Imroved heavy water reactor efficiency, energy and Fissonium Flux yield</t>
-  </si>
-  <si>
     <t>Improved Heavy Water Reactor</t>
   </si>
   <si>
@@ -5183,9 +5156,6 @@
     <t>gui/menu/research/description/morphium_factory_lvl_3</t>
   </si>
   <si>
-    <t>We found a way to synthetically replicate Morphium utilizing special fragments of the Xmorph tech. We still do not fully understand how they work, but that can be saved for later</t>
-  </si>
-  <si>
     <t>gui/hud/building_description/morphium_factory</t>
   </si>
   <si>
@@ -5490,6 +5460,36 @@
   </si>
   <si>
     <t>Provides detailed mappings of underground deposits. This increases yield of nearby geothermal &amp; gas and liquid extractors</t>
+  </si>
+  <si>
+    <t>These walls automatically recede into the ground when the Mech is close to them. This allows the user to shoot over them with ease and negates the need for building gates. Resistant to area and acid damage but very fragile to fire damage. The walls also regenerate missing hit points over time but do not reconstruct from ruins by themselves.</t>
+  </si>
+  <si>
+    <t>Improved heavy water reactor efficiency &amp; energy and Fissonium Flux yield</t>
+  </si>
+  <si>
+    <t>We found a way to synthetically replicate Morphium utilizing special fragments of the Xmorph tech. We still do not fully understand how they work but that can be saved for later</t>
+  </si>
+  <si>
+    <t>More advanced version of the Drone Attack Tower with more drones which shoot rocket propelled explosives</t>
+  </si>
+  <si>
+    <t>More advanced version of the Drone Attack Tower with more drones that shoot incindiary ammunition</t>
+  </si>
+  <si>
+    <t>More advanced version of the Drone Attack Tower with more drones that shoot cryogenic high caliber ammunition</t>
+  </si>
+  <si>
+    <t>More advanced version of the Drone Attack Tower with more drones that attack via lighting strikes</t>
+  </si>
+  <si>
+    <t>A silo housing a massive rocket launched vertically and aimed at distant targets. Once the rocket reaches destination it releases multiple explosive devices that cover a very large area with acidic substance</t>
+  </si>
+  <si>
+    <t>A silo housing a massive rocket launched vertically and aimed at distant targets. Once the rocket reaches destination it releases multiple explosive devices that cover a very large area with a cryogenic shock</t>
+  </si>
+  <si>
+    <t>Provides basic protection for the base. Can be built in multiple layers. Cheap reliable and sturdy.</t>
   </si>
 </sst>
 </file>
@@ -6376,66 +6376,66 @@
     </row>
     <row r="2" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>1819</v>
+        <v>1809</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1820</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>1645</v>
+        <v>1639</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1647</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>1642</v>
+        <v>1636</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>1643</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>1644</v>
+        <v>1638</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>1646</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>1262</v>
+        <v>1260</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>1282</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>1265</v>
+        <v>1263</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>1285</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>1263</v>
+        <v>1261</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>1283</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>1284</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6443,7 +6443,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>1388</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6451,7 +6451,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>1389</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6459,7 +6459,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1390</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6467,7 +6467,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>1395</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6483,12 +6483,12 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>1391</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>1401</v>
+        <v>1399</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>15</v>
@@ -6496,26 +6496,26 @@
     </row>
     <row r="17" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>1472</v>
+        <v>1470</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>1477</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>1471</v>
+        <v>1469</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>1473</v>
+        <v>1471</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>1477</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6523,15 +6523,15 @@
         <v>16</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>1396</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>1402</v>
+        <v>1400</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>1403</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6539,7 +6539,7 @@
         <v>17</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>1393</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6547,7 +6547,7 @@
         <v>520</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>1392</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6555,7 +6555,7 @@
         <v>18</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>1397</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6563,12 +6563,12 @@
         <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>1394</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>1399</v>
+        <v>1397</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>20</v>
@@ -6576,26 +6576,26 @@
     </row>
     <row r="27" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>1470</v>
+        <v>1468</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>1476</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>1469</v>
+        <v>1467</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>1475</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
+        <v>1472</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>1474</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>1476</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6603,15 +6603,15 @@
         <v>21</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>1400</v>
+        <v>1398</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6691,7 +6691,7 @@
         <v>34</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>1204</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6707,7 +6707,7 @@
         <v>37</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6715,7 +6715,7 @@
         <v>38</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6768,18 +6768,18 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>1243</v>
+        <v>1241</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>1242</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6795,23 +6795,23 @@
         <v>871</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6819,23 +6819,23 @@
         <v>870</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6843,23 +6843,23 @@
         <v>874</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6867,23 +6867,23 @@
         <v>872</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6939,10 +6939,10 @@
     </row>
     <row r="72" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>1490</v>
+        <v>1488</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>1491</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6955,18 +6955,18 @@
     </row>
     <row r="74" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>1816</v>
+        <v>1806</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>1821</v>
+        <v>1811</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>1314</v>
+        <v>1312</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6979,10 +6979,10 @@
     </row>
     <row r="77" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>1664</v>
+        <v>1658</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>1687</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7003,15 +7003,15 @@
     </row>
     <row r="80" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>1741</v>
+        <v>1731</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>1754</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>1559</v>
+        <v>1557</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>621</v>
@@ -7019,7 +7019,7 @@
     </row>
     <row r="82" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>1560</v>
+        <v>1558</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>619</v>
@@ -7027,7 +7027,7 @@
     </row>
     <row r="83" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>1561</v>
+        <v>1559</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>620</v>
@@ -7062,18 +7062,18 @@
     </row>
     <row r="87" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>1421</v>
+        <v>1419</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>1427</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>1424</v>
+        <v>1422</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>1428</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.35">
@@ -7081,7 +7081,7 @@
         <v>269</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>1435</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.35">
@@ -7089,7 +7089,7 @@
         <v>278</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>1436</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.35">
@@ -7097,23 +7097,23 @@
         <v>279</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>1437</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>1547</v>
+        <v>1545</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>1543</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>1720</v>
+        <v>1710</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>1722</v>
+        <v>1712</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
@@ -7145,7 +7145,7 @@
         <v>50</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>1764</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7153,7 +7153,7 @@
         <v>51</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>1764</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7161,47 +7161,47 @@
         <v>52</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>1764</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>1761</v>
+        <v>1751</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>1767</v>
+        <v>1757</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
+        <v>1220</v>
+      </c>
+      <c r="B101" s="1" t="s">
         <v>1222</v>
-      </c>
-      <c r="B101" s="1" t="s">
-        <v>1224</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>1237</v>
+        <v>1235</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>1432</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>1238</v>
+        <v>1236</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>1433</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>1239</v>
+        <v>1237</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>1434</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7222,18 +7222,18 @@
     </row>
     <row r="107" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>1343</v>
+        <v>1341</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>1489</v>
+        <v>1487</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>1492</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7297,26 +7297,26 @@
     </row>
     <row r="116" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>1292</v>
+        <v>1290</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>1295</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>1512</v>
+        <v>1510</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>1510</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>1700</v>
+        <v>1691</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>1712</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7345,18 +7345,18 @@
     </row>
     <row r="122" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>1632</v>
+        <v>1626</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>1637</v>
+        <v>1631</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>1633</v>
+        <v>1627</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>1638</v>
+        <v>1632</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7479,23 +7479,23 @@
         <v>57</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>1289</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="139" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>1235</v>
+        <v>1233</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>1290</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="140" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>1236</v>
+        <v>1234</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>1291</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="141" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7540,10 +7540,10 @@
     </row>
     <row r="146" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>1325</v>
+        <v>1323</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7628,90 +7628,90 @@
     </row>
     <row r="157" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>1613</v>
+        <v>1607</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>1618</v>
+        <v>1612</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>1594</v>
+        <v>1588</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>1581</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>1595</v>
+        <v>1589</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>1580</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
-        <v>1596</v>
+        <v>1590</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>1593</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>1597</v>
+        <v>1591</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>1578</v>
+        <v>1572</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
-        <v>1598</v>
+        <v>1592</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>1579</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
-        <v>1614</v>
+        <v>1608</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>1619</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
-        <v>1696</v>
+        <v>1687</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>1692</v>
+        <v>1683</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>1648</v>
+        <v>1642</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>1674</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>1650</v>
+        <v>1644</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>1675</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>1358</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7732,10 +7732,10 @@
     </row>
     <row r="170" spans="1:2" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7860,31 +7860,31 @@
     </row>
     <row r="186" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="187" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="188" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B188" s="1" t="s">
         <v>1109</v>
-      </c>
-      <c r="B188" s="1" t="s">
-        <v>1110</v>
       </c>
     </row>
     <row r="189" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="B189" s="1" t="s">
         <v>1097</v>
@@ -7892,66 +7892,66 @@
     </row>
     <row r="190" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="191" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="192" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>1098</v>
+        <v>1821</v>
       </c>
     </row>
     <row r="193" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>1114</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="196" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="197" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="198" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7964,34 +7964,34 @@
     </row>
     <row r="199" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
-        <v>1258</v>
+        <v>1256</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="200" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
-        <v>1261</v>
+        <v>1259</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>1275</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="201" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
-        <v>1259</v>
+        <v>1257</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>1273</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="202" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
-        <v>1260</v>
+        <v>1258</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>1274</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="203" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -7999,7 +7999,7 @@
         <v>66</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>1404</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="204" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8007,7 +8007,7 @@
         <v>67</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>1405</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="205" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8015,7 +8015,7 @@
         <v>68</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>1406</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="206" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8023,7 +8023,7 @@
         <v>69</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>1407</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="207" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8039,12 +8039,12 @@
         <v>70</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>1408</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="209" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
-        <v>1416</v>
+        <v>1414</v>
       </c>
       <c r="B209" s="1" t="s">
         <v>71</v>
@@ -8052,26 +8052,26 @@
     </row>
     <row r="210" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
-        <v>1480</v>
+        <v>1478</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>1486</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="211" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
-        <v>1479</v>
+        <v>1477</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>1487</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="212" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
-        <v>1483</v>
+        <v>1481</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>1486</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="213" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8079,15 +8079,15 @@
         <v>72</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>1409</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="214" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
-        <v>1418</v>
+        <v>1416</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>1419</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="215" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8095,7 +8095,7 @@
         <v>73</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>1410</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="216" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8103,7 +8103,7 @@
         <v>521</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>1411</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="217" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8111,7 +8111,7 @@
         <v>74</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>1412</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="218" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8119,12 +8119,12 @@
         <v>75</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>1413</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="219" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
-        <v>1415</v>
+        <v>1413</v>
       </c>
       <c r="B219" s="1" t="s">
         <v>76</v>
@@ -8132,26 +8132,26 @@
     </row>
     <row r="220" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
-        <v>1482</v>
+        <v>1480</v>
       </c>
       <c r="B220" s="1" t="s">
-        <v>1485</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="221" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
-        <v>1481</v>
+        <v>1479</v>
       </c>
       <c r="B221" s="1" t="s">
-        <v>1488</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="222" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
-        <v>1484</v>
+        <v>1482</v>
       </c>
       <c r="B222" s="1" t="s">
-        <v>1485</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="223" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8159,15 +8159,15 @@
         <v>77</v>
       </c>
       <c r="B223" s="1" t="s">
-        <v>1414</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="224" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
-        <v>1417</v>
+        <v>1415</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>1420</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="225" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8316,10 +8316,10 @@
     </row>
     <row r="243" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
-        <v>1241</v>
+        <v>1239</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>1240</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="244" spans="1:3" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8437,18 +8437,18 @@
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
-        <v>1817</v>
+        <v>1807</v>
       </c>
       <c r="B257" s="1" t="s">
-        <v>1818</v>
+        <v>1808</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
-        <v>1315</v>
+        <v>1313</v>
       </c>
       <c r="B258" s="1" t="s">
-        <v>1328</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.35">
@@ -8461,42 +8461,42 @@
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
-        <v>1665</v>
+        <v>1659</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>1686</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
-        <v>1742</v>
+        <v>1732</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>1748</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
-        <v>1553</v>
+        <v>1551</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>1556</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
-        <v>1554</v>
+        <v>1552</v>
       </c>
       <c r="B263" s="1" t="s">
-        <v>1557</v>
+        <v>1555</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
-        <v>1555</v>
+        <v>1553</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>1558</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.35">
@@ -8528,18 +8528,18 @@
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
-        <v>1422</v>
+        <v>1420</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>1425</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
-        <v>1423</v>
+        <v>1421</v>
       </c>
       <c r="B269" s="1" t="s">
-        <v>1426</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.35">
@@ -8568,21 +8568,21 @@
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
-        <v>1548</v>
+        <v>1546</v>
       </c>
       <c r="B273" s="1" t="s">
-        <v>1541</v>
+        <v>1539</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>1545</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
-        <v>1721</v>
+        <v>1711</v>
       </c>
       <c r="B274" s="1" t="s">
-        <v>1737</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.35">
@@ -8619,42 +8619,42 @@
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
-        <v>1762</v>
+        <v>1752</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>1763</v>
+        <v>1753</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
+        <v>1219</v>
+      </c>
+      <c r="B280" s="1" t="s">
         <v>1221</v>
-      </c>
-      <c r="B280" s="1" t="s">
-        <v>1223</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
       <c r="B281" s="1" t="s">
-        <v>1429</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>1430</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
-        <v>1288</v>
+        <v>1286</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>1431</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.35">
@@ -8667,10 +8667,10 @@
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
-        <v>1344</v>
+        <v>1342</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>1345</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.35">
@@ -8719,26 +8719,26 @@
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
-        <v>1293</v>
+        <v>1291</v>
       </c>
       <c r="B290" s="1" t="s">
-        <v>1294</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
-        <v>1513</v>
+        <v>1511</v>
       </c>
       <c r="B291" s="1" t="s">
-        <v>1514</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
-        <v>1701</v>
+        <v>1692</v>
       </c>
       <c r="B292" s="1" t="s">
-        <v>1711</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.35">
@@ -8767,18 +8767,18 @@
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
+        <v>1624</v>
+      </c>
+      <c r="B296" s="1" t="s">
         <v>1630</v>
-      </c>
-      <c r="B296" s="1" t="s">
-        <v>1636</v>
       </c>
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
-        <v>1631</v>
+        <v>1625</v>
       </c>
       <c r="B297" s="1" t="s">
-        <v>1641</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.35">
@@ -8903,10 +8903,10 @@
     </row>
     <row r="313" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="B313" s="1" t="s">
-        <v>1329</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="314" spans="1:2" x14ac:dyDescent="0.35">
@@ -9007,90 +9007,90 @@
     </row>
     <row r="326" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
-        <v>1612</v>
+        <v>1606</v>
       </c>
       <c r="B326" s="1" t="s">
-        <v>1616</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="327" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
-        <v>1599</v>
+        <v>1593</v>
       </c>
       <c r="B327" s="1" t="s">
-        <v>1565</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="328" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
-        <v>1600</v>
+        <v>1594</v>
       </c>
       <c r="B328" s="1" t="s">
-        <v>1564</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="329" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
-        <v>1601</v>
+        <v>1595</v>
       </c>
       <c r="B329" s="1" t="s">
-        <v>1592</v>
+        <v>1586</v>
       </c>
     </row>
     <row r="330" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
-        <v>1602</v>
+        <v>1596</v>
       </c>
       <c r="B330" s="1" t="s">
-        <v>1562</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="331" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
-        <v>1603</v>
+        <v>1597</v>
       </c>
       <c r="B331" s="1" t="s">
-        <v>1563</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="332" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
-        <v>1615</v>
+        <v>1609</v>
       </c>
       <c r="B332" s="1" t="s">
-        <v>1617</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="333" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
-        <v>1695</v>
+        <v>1686</v>
       </c>
       <c r="B333" s="1" t="s">
-        <v>1691</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="334" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
-        <v>1649</v>
+        <v>1643</v>
       </c>
       <c r="B334" s="1" t="s">
-        <v>1672</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="335" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
-        <v>1651</v>
+        <v>1645</v>
       </c>
       <c r="B335" s="1" t="s">
-        <v>1673</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="336" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
       <c r="B336" s="1" t="s">
-        <v>1357</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="337" spans="1:2" x14ac:dyDescent="0.35">
@@ -9111,10 +9111,10 @@
     </row>
     <row r="339" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
       <c r="B339" s="1" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="340" spans="1:2" x14ac:dyDescent="0.35">
@@ -9247,66 +9247,66 @@
     </row>
     <row r="356" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A356" t="s">
-        <v>1438</v>
+        <v>1436</v>
       </c>
       <c r="B356" s="1" t="s">
-        <v>1439</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="357" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
-        <v>1440</v>
+        <v>1438</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>1441</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="358" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
-        <v>1442</v>
+        <v>1440</v>
       </c>
       <c r="B358" s="1" t="s">
-        <v>1443</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="359" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
-        <v>1444</v>
+        <v>1442</v>
       </c>
       <c r="B359" s="1" t="s">
-        <v>1445</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="360" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
-        <v>1446</v>
+        <v>1444</v>
       </c>
       <c r="B360" s="1" t="s">
-        <v>1447</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="361" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
-        <v>1448</v>
+        <v>1446</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>1449</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="362" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
-        <v>1450</v>
+        <v>1448</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>1451</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="363" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
-        <v>1452</v>
+        <v>1450</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>1453</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="364" spans="1:2" x14ac:dyDescent="0.35">
@@ -9383,10 +9383,10 @@
     </row>
     <row r="373" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A373" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
       <c r="B373" s="1" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="374" spans="1:2" x14ac:dyDescent="0.35">
@@ -9415,26 +9415,26 @@
     </row>
     <row r="377" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A377" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
       <c r="B377" s="1" t="s">
-        <v>1280</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="378" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B378" s="1" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="379" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
-        <v>1270</v>
+        <v>1268</v>
       </c>
       <c r="B379" s="1" t="s">
-        <v>1281</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="380" spans="1:2" x14ac:dyDescent="0.35">
@@ -9442,15 +9442,15 @@
         <v>505</v>
       </c>
       <c r="B380" s="1" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="381" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="B381" s="1" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="382" spans="1:2" x14ac:dyDescent="0.35">
@@ -9458,7 +9458,7 @@
         <v>506</v>
       </c>
       <c r="B382" s="1" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="383" spans="1:2" x14ac:dyDescent="0.35">
@@ -9466,23 +9466,23 @@
         <v>652</v>
       </c>
       <c r="B383" s="1" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="384" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
-        <v>1591</v>
+        <v>1585</v>
       </c>
       <c r="B384" s="1" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="385" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A385" t="s">
-        <v>1535</v>
+        <v>1533</v>
       </c>
       <c r="B385" s="1" t="s">
-        <v>1536</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="386" spans="1:2" x14ac:dyDescent="0.35">
@@ -9490,15 +9490,15 @@
         <v>507</v>
       </c>
       <c r="B386" s="1" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="387" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A387" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="B387" s="1" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="388" spans="1:2" x14ac:dyDescent="0.35">
@@ -9506,7 +9506,7 @@
         <v>508</v>
       </c>
       <c r="B388" s="1" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="389" spans="1:2" x14ac:dyDescent="0.35">
@@ -9514,15 +9514,15 @@
         <v>653</v>
       </c>
       <c r="B389" s="1" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="390" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A390" t="s">
-        <v>1590</v>
+        <v>1584</v>
       </c>
       <c r="B390" s="1" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="391" spans="1:2" x14ac:dyDescent="0.35">
@@ -9530,15 +9530,15 @@
         <v>509</v>
       </c>
       <c r="B391" s="1" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="392" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A392" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="393" spans="1:2" x14ac:dyDescent="0.35">
@@ -9546,7 +9546,7 @@
         <v>510</v>
       </c>
       <c r="B393" s="1" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="394" spans="1:2" x14ac:dyDescent="0.35">
@@ -9554,15 +9554,15 @@
         <v>654</v>
       </c>
       <c r="B394" s="1" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="395" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
-        <v>1582</v>
+        <v>1576</v>
       </c>
       <c r="B395" s="1" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="396" spans="1:2" x14ac:dyDescent="0.35">
@@ -9570,15 +9570,15 @@
         <v>511</v>
       </c>
       <c r="B396" s="1" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="397" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A397" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
       <c r="B397" s="1" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="398" spans="1:2" x14ac:dyDescent="0.35">
@@ -9586,7 +9586,7 @@
         <v>512</v>
       </c>
       <c r="B398" s="1" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="399" spans="1:2" x14ac:dyDescent="0.35">
@@ -9594,15 +9594,15 @@
         <v>655</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="400" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
-        <v>1583</v>
+        <v>1577</v>
       </c>
       <c r="B400" s="1" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="401" spans="1:2" x14ac:dyDescent="0.35">
@@ -9610,15 +9610,15 @@
         <v>513</v>
       </c>
       <c r="B401" s="1" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="402" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="B402" s="1" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="403" spans="1:2" x14ac:dyDescent="0.35">
@@ -9626,7 +9626,7 @@
         <v>514</v>
       </c>
       <c r="B403" s="1" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="404" spans="1:2" x14ac:dyDescent="0.35">
@@ -9634,23 +9634,23 @@
         <v>656</v>
       </c>
       <c r="B404" s="1" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="405" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
-        <v>1584</v>
+        <v>1578</v>
       </c>
       <c r="B405" s="1" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="406" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
-        <v>1533</v>
+        <v>1531</v>
       </c>
       <c r="B406" s="1" t="s">
-        <v>1534</v>
+        <v>1532</v>
       </c>
     </row>
     <row r="407" spans="1:2" x14ac:dyDescent="0.35">
@@ -9695,18 +9695,18 @@
     </row>
     <row r="412" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A412" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="B412" s="1" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="413" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A413" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="B413" s="1" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="414" spans="1:2" x14ac:dyDescent="0.35">
@@ -9719,18 +9719,18 @@
     </row>
     <row r="415" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
       <c r="B415" s="1" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="416" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A416" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="B416" s="1" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="417" spans="1:2" x14ac:dyDescent="0.35">
@@ -9791,18 +9791,18 @@
     </row>
     <row r="424" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A424" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="B424" s="1" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="425" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A425" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="B425" s="1" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="426" spans="1:2" x14ac:dyDescent="0.35">
@@ -9815,18 +9815,18 @@
     </row>
     <row r="427" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A427" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="B427" s="1" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="428" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A428" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="B428" s="1" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="429" spans="1:2" x14ac:dyDescent="0.35">
@@ -9866,15 +9866,15 @@
         <v>1072</v>
       </c>
       <c r="B433" s="1" t="s">
-        <v>1525</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="434" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
-        <v>1518</v>
+        <v>1516</v>
       </c>
       <c r="B434" s="1" t="s">
-        <v>1524</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="435" spans="1:2" x14ac:dyDescent="0.35">
@@ -9890,15 +9890,15 @@
         <v>570</v>
       </c>
       <c r="B436" s="1" t="s">
-        <v>1526</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="437" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
-        <v>1522</v>
+        <v>1520</v>
       </c>
       <c r="B437" s="1" t="s">
-        <v>1523</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="438" spans="1:2" x14ac:dyDescent="0.35">
@@ -10007,10 +10007,10 @@
     </row>
     <row r="451" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A451" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B451" s="1" t="s">
         <v>1308</v>
-      </c>
-      <c r="B451" s="1" t="s">
-        <v>1310</v>
       </c>
     </row>
     <row r="452" spans="1:2" x14ac:dyDescent="0.35">
@@ -10018,7 +10018,7 @@
         <v>868</v>
       </c>
       <c r="B452" s="1" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="453" spans="1:2" x14ac:dyDescent="0.35">
@@ -10026,7 +10026,7 @@
         <v>890</v>
       </c>
       <c r="B453" s="1" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="454" spans="1:2" x14ac:dyDescent="0.35">
@@ -10034,7 +10034,7 @@
         <v>894</v>
       </c>
       <c r="B454" s="1" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="455" spans="1:2" x14ac:dyDescent="0.35">
@@ -10042,7 +10042,7 @@
         <v>867</v>
       </c>
       <c r="B455" s="1" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="456" spans="1:2" x14ac:dyDescent="0.35">
@@ -10050,7 +10050,7 @@
         <v>891</v>
       </c>
       <c r="B456" s="1" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="457" spans="1:2" x14ac:dyDescent="0.35">
@@ -10058,7 +10058,7 @@
         <v>895</v>
       </c>
       <c r="B457" s="1" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="458" spans="1:2" x14ac:dyDescent="0.35">
@@ -10066,7 +10066,7 @@
         <v>873</v>
       </c>
       <c r="B458" s="1" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="459" spans="1:2" x14ac:dyDescent="0.35">
@@ -10074,7 +10074,7 @@
         <v>892</v>
       </c>
       <c r="B459" s="1" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="460" spans="1:2" x14ac:dyDescent="0.35">
@@ -10082,7 +10082,7 @@
         <v>896</v>
       </c>
       <c r="B460" s="1" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="461" spans="1:2" x14ac:dyDescent="0.35">
@@ -10090,7 +10090,7 @@
         <v>869</v>
       </c>
       <c r="B461" s="1" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="462" spans="1:2" x14ac:dyDescent="0.35">
@@ -10098,7 +10098,7 @@
         <v>893</v>
       </c>
       <c r="B462" s="1" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="463" spans="1:2" x14ac:dyDescent="0.35">
@@ -10106,63 +10106,63 @@
         <v>897</v>
       </c>
       <c r="B463" s="1" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="464" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A464" t="s">
-        <v>1212</v>
+        <v>1210</v>
       </c>
       <c r="B464" s="1" t="s">
-        <v>1218</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="465" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A465" t="s">
-        <v>1213</v>
+        <v>1211</v>
       </c>
       <c r="B465" s="1" t="s">
-        <v>1219</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="466" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A466" t="s">
-        <v>1214</v>
+        <v>1212</v>
       </c>
       <c r="B466" s="1" t="s">
-        <v>1220</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="467" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A467" t="s">
-        <v>1454</v>
+        <v>1452</v>
       </c>
       <c r="B467" s="1" t="s">
-        <v>1460</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="468" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A468" t="s">
-        <v>1462</v>
+        <v>1460</v>
       </c>
       <c r="B468" s="1" t="s">
-        <v>1467</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="469" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A469" t="s">
+        <v>1455</v>
+      </c>
+      <c r="B469" s="1" t="s">
         <v>1457</v>
-      </c>
-      <c r="B469" s="1" t="s">
-        <v>1459</v>
       </c>
     </row>
     <row r="470" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A470" t="s">
-        <v>1468</v>
+        <v>1466</v>
       </c>
       <c r="B470" s="1" t="s">
-        <v>1467</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="471" spans="1:2" x14ac:dyDescent="0.35">
@@ -10202,7 +10202,7 @@
         <v>1068</v>
       </c>
       <c r="B475" s="1" t="s">
-        <v>1516</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="476" spans="1:2" x14ac:dyDescent="0.35">
@@ -10231,50 +10231,50 @@
     </row>
     <row r="479" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A479" t="s">
-        <v>1797</v>
+        <v>1787</v>
       </c>
       <c r="B479" s="1" t="s">
-        <v>1814</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="480" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A480" t="s">
-        <v>1789</v>
+        <v>1779</v>
       </c>
       <c r="B480" s="1" t="s">
-        <v>1813</v>
+        <v>1803</v>
       </c>
     </row>
     <row r="481" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A481" t="s">
-        <v>1790</v>
+        <v>1780</v>
       </c>
       <c r="B481" s="1" t="s">
-        <v>1815</v>
+        <v>1805</v>
       </c>
     </row>
     <row r="482" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A482" t="s">
-        <v>1794</v>
+        <v>1784</v>
       </c>
       <c r="B482" s="1" t="s">
-        <v>1801</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="483" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A483" t="s">
-        <v>1772</v>
+        <v>1762</v>
       </c>
       <c r="B483" s="1" t="s">
-        <v>1811</v>
+        <v>1801</v>
       </c>
     </row>
     <row r="484" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A484" t="s">
-        <v>1773</v>
+        <v>1763</v>
       </c>
       <c r="B484" s="1" t="s">
-        <v>1812</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="485" spans="1:2" x14ac:dyDescent="0.35">
@@ -10287,58 +10287,58 @@
     </row>
     <row r="486" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A486" t="s">
-        <v>1316</v>
+        <v>1314</v>
       </c>
       <c r="B486" s="1" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="487" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A487" t="s">
-        <v>1317</v>
+        <v>1315</v>
       </c>
       <c r="B487" s="1" t="s">
-        <v>1323</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="488" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A488" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
       <c r="B488" s="1" t="s">
-        <v>1324</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="489" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A489" t="s">
-        <v>1662</v>
+        <v>1656</v>
       </c>
       <c r="B489" s="1" t="s">
-        <v>1684</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="490" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A490" t="s">
-        <v>1663</v>
+        <v>1657</v>
       </c>
       <c r="B490" s="1" t="s">
-        <v>1685</v>
+        <v>1677</v>
       </c>
     </row>
     <row r="491" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A491" t="s">
-        <v>1666</v>
+        <v>1660</v>
       </c>
       <c r="B491" s="1" t="s">
-        <v>1688</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="492" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A492" t="s">
-        <v>1667</v>
+        <v>1661</v>
       </c>
       <c r="B492" s="1" t="s">
-        <v>1689</v>
+        <v>1813</v>
       </c>
     </row>
     <row r="493" spans="1:2" x14ac:dyDescent="0.35">
@@ -10383,26 +10383,26 @@
     </row>
     <row r="498" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A498" t="s">
-        <v>1752</v>
+        <v>1742</v>
       </c>
       <c r="B498" s="1" t="s">
-        <v>1753</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="499" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A499" t="s">
-        <v>1746</v>
+        <v>1736</v>
       </c>
       <c r="B499" s="1" t="s">
-        <v>1753</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="500" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A500" t="s">
-        <v>1747</v>
+        <v>1737</v>
       </c>
       <c r="B500" s="1" t="s">
-        <v>1753</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="501" spans="1:2" x14ac:dyDescent="0.35">
@@ -10647,98 +10647,98 @@
     </row>
     <row r="531" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A531" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
       <c r="B531" s="1" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="532" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A532" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
       <c r="B532" s="1" t="s">
-        <v>1252</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="533" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A533" t="s">
-        <v>1251</v>
+        <v>1249</v>
       </c>
       <c r="B533" s="1" t="s">
-        <v>1255</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="534" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A534" t="s">
+        <v>1492</v>
+      </c>
+      <c r="B534" s="1" t="s">
         <v>1494</v>
-      </c>
-      <c r="B534" s="1" t="s">
-        <v>1496</v>
       </c>
     </row>
     <row r="535" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A535" t="s">
-        <v>1499</v>
+        <v>1497</v>
       </c>
       <c r="B535" s="1" t="s">
-        <v>1505</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="536" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A536" t="s">
-        <v>1500</v>
+        <v>1498</v>
       </c>
       <c r="B536" s="1" t="s">
-        <v>1506</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="537" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A537" t="s">
-        <v>1501</v>
+        <v>1499</v>
       </c>
       <c r="B537" s="1" t="s">
-        <v>1507</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="538" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A538" t="s">
-        <v>1549</v>
+        <v>1547</v>
       </c>
       <c r="B538" s="1" t="s">
-        <v>1543</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="539" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A539" t="s">
-        <v>1550</v>
+        <v>1548</v>
       </c>
       <c r="B539" s="1" t="s">
-        <v>1544</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="540" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A540" t="s">
-        <v>1716</v>
+        <v>1707</v>
       </c>
       <c r="B540" s="1" t="s">
-        <v>1719</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="541" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A541" t="s">
-        <v>1717</v>
+        <v>1708</v>
       </c>
       <c r="B541" s="1" t="s">
-        <v>1724</v>
+        <v>1714</v>
       </c>
     </row>
     <row r="542" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A542" t="s">
-        <v>1718</v>
+        <v>1709</v>
       </c>
       <c r="B542" s="1" t="s">
-        <v>1723</v>
+        <v>1713</v>
       </c>
     </row>
     <row r="543" spans="1:2" x14ac:dyDescent="0.35">
@@ -10746,7 +10746,7 @@
         <v>1058</v>
       </c>
       <c r="B543" s="1" t="s">
-        <v>1530</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="544" spans="1:2" x14ac:dyDescent="0.35">
@@ -10754,31 +10754,31 @@
         <v>1059</v>
       </c>
       <c r="B544" s="1" t="s">
-        <v>1531</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="545" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
-        <v>1527</v>
+        <v>1525</v>
       </c>
       <c r="B545" s="1" t="s">
-        <v>1532</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="546" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A546" t="s">
-        <v>1759</v>
+        <v>1749</v>
       </c>
       <c r="B546" s="1" t="s">
-        <v>1767</v>
+        <v>1757</v>
       </c>
     </row>
     <row r="547" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A547" t="s">
-        <v>1760</v>
+        <v>1750</v>
       </c>
       <c r="B547" s="1" t="s">
-        <v>1768</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="548" spans="1:2" x14ac:dyDescent="0.35">
@@ -10807,26 +10807,26 @@
     </row>
     <row r="551" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A551" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="B551" s="1" t="s">
-        <v>1234</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="552" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A552" t="s">
-        <v>1229</v>
+        <v>1227</v>
       </c>
       <c r="B552" s="1" t="s">
-        <v>1234</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="553" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A553" t="s">
-        <v>1230</v>
+        <v>1228</v>
       </c>
       <c r="B553" s="1" t="s">
-        <v>1234</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="554" spans="1:2" x14ac:dyDescent="0.35">
@@ -10887,26 +10887,26 @@
     </row>
     <row r="561" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A561" t="s">
-        <v>1334</v>
+        <v>1332</v>
       </c>
       <c r="B561" s="1" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="562" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A562" t="s">
-        <v>1335</v>
+        <v>1333</v>
       </c>
       <c r="B562" s="1" t="s">
-        <v>1341</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="563" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A563" t="s">
-        <v>1336</v>
+        <v>1334</v>
       </c>
       <c r="B563" s="1" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="564" spans="1:2" x14ac:dyDescent="0.35">
@@ -10967,58 +10967,58 @@
     </row>
     <row r="571" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A571" t="s">
-        <v>1306</v>
+        <v>1304</v>
       </c>
       <c r="B571" s="1" t="s">
-        <v>1302</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="572" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A572" t="s">
-        <v>1304</v>
+        <v>1302</v>
       </c>
       <c r="B572" s="1" t="s">
-        <v>1303</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="573" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A573" t="s">
-        <v>1305</v>
+        <v>1303</v>
       </c>
       <c r="B573" s="1" t="s">
-        <v>1303</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="574" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A574" t="s">
+        <v>1507</v>
+      </c>
+      <c r="B574" s="1" t="s">
         <v>1509</v>
-      </c>
-      <c r="B574" s="1" t="s">
-        <v>1511</v>
       </c>
     </row>
     <row r="575" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A575" t="s">
-        <v>1705</v>
+        <v>1696</v>
       </c>
       <c r="B575" s="1" t="s">
-        <v>1708</v>
+        <v>1699</v>
       </c>
     </row>
     <row r="576" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A576" t="s">
-        <v>1706</v>
+        <v>1697</v>
       </c>
       <c r="B576" s="1" t="s">
-        <v>1709</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="577" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A577" t="s">
-        <v>1707</v>
+        <v>1698</v>
       </c>
       <c r="B577" s="1" t="s">
-        <v>1710</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="578" spans="1:2" x14ac:dyDescent="0.35">
@@ -11047,18 +11047,18 @@
     </row>
     <row r="581" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A581" t="s">
-        <v>1628</v>
+        <v>1622</v>
       </c>
       <c r="B581" s="1" t="s">
-        <v>1639</v>
+        <v>1633</v>
       </c>
     </row>
     <row r="582" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A582" t="s">
-        <v>1629</v>
+        <v>1623</v>
       </c>
       <c r="B582" s="1" t="s">
-        <v>1640</v>
+        <v>1634</v>
       </c>
     </row>
     <row r="583" spans="1:2" x14ac:dyDescent="0.35">
@@ -11087,26 +11087,26 @@
     </row>
     <row r="586" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A586" t="s">
-        <v>1795</v>
+        <v>1785</v>
       </c>
       <c r="B586" s="1" t="s">
-        <v>1807</v>
+        <v>1797</v>
       </c>
     </row>
     <row r="587" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A587" t="s">
-        <v>1777</v>
+        <v>1767</v>
       </c>
       <c r="B587" s="1" t="s">
-        <v>1808</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="588" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A588" t="s">
-        <v>1778</v>
+        <v>1768</v>
       </c>
       <c r="B588" s="1" t="s">
-        <v>1807</v>
+        <v>1797</v>
       </c>
     </row>
     <row r="589" spans="1:2" x14ac:dyDescent="0.35">
@@ -11183,58 +11183,58 @@
     </row>
     <row r="598" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A598" t="s">
-        <v>1658</v>
+        <v>1652</v>
       </c>
       <c r="B598" s="1" t="s">
-        <v>1681</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="599" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A599" t="s">
-        <v>1659</v>
+        <v>1653</v>
       </c>
       <c r="B599" s="1" t="s">
-        <v>1681</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="600" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A600" t="s">
-        <v>1656</v>
+        <v>1650</v>
       </c>
       <c r="B600" s="1" t="s">
-        <v>1680</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="601" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A601" t="s">
-        <v>1657</v>
+        <v>1651</v>
       </c>
       <c r="B601" s="1" t="s">
-        <v>1680</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="602" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A602" t="s">
-        <v>1354</v>
+        <v>1352</v>
       </c>
       <c r="B602" s="1" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="603" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A603" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="B603" s="1" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="604" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A604" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="B604" s="1" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="605" spans="1:2" x14ac:dyDescent="0.35">
@@ -11271,74 +11271,74 @@
     </row>
     <row r="609" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A609" t="s">
-        <v>1609</v>
+        <v>1603</v>
       </c>
       <c r="B609" s="1" t="s">
-        <v>1623</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="610" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A610" t="s">
-        <v>1608</v>
+        <v>1602</v>
       </c>
       <c r="B610" s="1" t="s">
-        <v>1624</v>
+        <v>1618</v>
       </c>
     </row>
     <row r="611" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A611" t="s">
-        <v>1573</v>
+        <v>1571</v>
       </c>
       <c r="B611" s="1" t="s">
-        <v>1574</v>
+        <v>1815</v>
       </c>
     </row>
     <row r="612" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A612" t="s">
-        <v>1572</v>
+        <v>1570</v>
       </c>
       <c r="B612" s="1" t="s">
-        <v>1575</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="613" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A613" t="s">
-        <v>1570</v>
+        <v>1568</v>
       </c>
       <c r="B613" s="1" t="s">
-        <v>1576</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="614" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A614" t="s">
-        <v>1571</v>
+        <v>1569</v>
       </c>
       <c r="B614" s="1" t="s">
-        <v>1577</v>
+        <v>1818</v>
       </c>
     </row>
     <row r="615" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A615" t="s">
-        <v>1611</v>
+        <v>1605</v>
       </c>
       <c r="B615" s="1" t="s">
-        <v>1622</v>
+        <v>1616</v>
       </c>
     </row>
     <row r="616" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A616" t="s">
-        <v>1610</v>
+        <v>1604</v>
       </c>
       <c r="B616" s="1" t="s">
-        <v>1625</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="617" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A617" t="s">
-        <v>1371</v>
+        <v>1369</v>
       </c>
       <c r="B617" s="1" t="s">
-        <v>1369</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="618" spans="1:2" x14ac:dyDescent="0.35">
@@ -11383,34 +11383,34 @@
     </row>
     <row r="623" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A623" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="B623" s="1" t="s">
-        <v>1385</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="624" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A624" t="s">
-        <v>1381</v>
+        <v>1379</v>
       </c>
       <c r="B624" s="1" t="s">
-        <v>1386</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="625" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A625" t="s">
+        <v>1380</v>
+      </c>
+      <c r="B625" s="1" t="s">
         <v>1382</v>
-      </c>
-      <c r="B625" s="1" t="s">
-        <v>1384</v>
       </c>
     </row>
     <row r="626" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A626" t="s">
-        <v>1383</v>
+        <v>1381</v>
       </c>
       <c r="B626" s="1" t="s">
-        <v>1387</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="627" spans="1:2" x14ac:dyDescent="0.35">
@@ -11455,26 +11455,26 @@
     </row>
     <row r="632" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A632" t="s">
+        <v>1786</v>
+      </c>
+      <c r="B632" s="1" t="s">
         <v>1796</v>
-      </c>
-      <c r="B632" s="1" t="s">
-        <v>1806</v>
       </c>
     </row>
     <row r="633" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A633" t="s">
-        <v>1782</v>
+        <v>1772</v>
       </c>
       <c r="B633" s="1" t="s">
-        <v>1809</v>
+        <v>1799</v>
       </c>
     </row>
     <row r="634" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A634" t="s">
-        <v>1783</v>
+        <v>1773</v>
       </c>
       <c r="B634" s="1" t="s">
-        <v>1810</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="635" spans="1:2" x14ac:dyDescent="0.35">
@@ -11503,26 +11503,26 @@
     </row>
     <row r="638" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A638" t="s">
-        <v>1268</v>
+        <v>1266</v>
       </c>
       <c r="B638" s="1" t="s">
-        <v>1278</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="639" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A639" t="s">
-        <v>1266</v>
+        <v>1264</v>
       </c>
       <c r="B639" s="1" t="s">
-        <v>1276</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="640" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A640" t="s">
-        <v>1267</v>
+        <v>1265</v>
       </c>
       <c r="B640" s="1" t="s">
-        <v>1277</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="641" spans="1:2" x14ac:dyDescent="0.35">
@@ -11535,10 +11535,10 @@
     </row>
     <row r="642" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A642" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="B642" s="1" t="s">
-        <v>1137</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="643" spans="1:2" x14ac:dyDescent="0.35">
@@ -11554,31 +11554,31 @@
         <v>646</v>
       </c>
       <c r="B644" s="1" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="645" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A645" t="s">
-        <v>1585</v>
+        <v>1579</v>
       </c>
       <c r="B645" s="1" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="646" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A646" t="s">
-        <v>1736</v>
+        <v>1726</v>
       </c>
       <c r="B646" s="1" t="s">
-        <v>1735</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="647" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A647" t="s">
-        <v>1537</v>
+        <v>1535</v>
       </c>
       <c r="B647" s="1" t="s">
-        <v>1540</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="648" spans="1:2" x14ac:dyDescent="0.35">
@@ -11591,10 +11591,10 @@
     </row>
     <row r="649" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A649" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="B649" s="1" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="650" spans="1:2" x14ac:dyDescent="0.35">
@@ -11610,15 +11610,15 @@
         <v>645</v>
       </c>
       <c r="B651" s="1" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="652" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
-        <v>1586</v>
+        <v>1580</v>
       </c>
       <c r="B652" s="1" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="653" spans="1:2" x14ac:dyDescent="0.35">
@@ -11631,10 +11631,10 @@
     </row>
     <row r="654" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="B654" s="1" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="655" spans="1:2" x14ac:dyDescent="0.35">
@@ -11650,15 +11650,15 @@
         <v>644</v>
       </c>
       <c r="B656" s="1" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="657" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1587</v>
+        <v>1581</v>
       </c>
       <c r="B657" s="1" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="658" spans="1:2" x14ac:dyDescent="0.35">
@@ -11671,10 +11671,10 @@
     </row>
     <row r="659" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="B659" s="1" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="660" spans="1:2" x14ac:dyDescent="0.35">
@@ -11690,15 +11690,15 @@
         <v>643</v>
       </c>
       <c r="B661" s="1" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="662" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1588</v>
+        <v>1582</v>
       </c>
       <c r="B662" s="1" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="663" spans="1:2" x14ac:dyDescent="0.35">
@@ -11711,10 +11711,10 @@
     </row>
     <row r="664" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A664" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="B664" s="1" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="665" spans="1:2" x14ac:dyDescent="0.35">
@@ -11730,23 +11730,23 @@
         <v>642</v>
       </c>
       <c r="B666" s="1" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="667" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A667" t="s">
-        <v>1589</v>
+        <v>1583</v>
       </c>
       <c r="B667" s="1" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="668" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A668" t="s">
-        <v>1538</v>
+        <v>1536</v>
       </c>
       <c r="B668" s="1" t="s">
-        <v>1539</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="669" spans="1:2" x14ac:dyDescent="0.35">
@@ -11791,18 +11791,18 @@
     </row>
     <row r="674" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A674" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="B674" s="1" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="675" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A675" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
       <c r="B675" s="1" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="676" spans="1:2" x14ac:dyDescent="0.35">
@@ -11815,18 +11815,18 @@
     </row>
     <row r="677" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A677" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="B677" s="1" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="678" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A678" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
       <c r="B678" s="1" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="679" spans="1:2" x14ac:dyDescent="0.35">
@@ -11887,18 +11887,18 @@
     </row>
     <row r="686" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A686" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="B686" s="1" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="687" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A687" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="B687" s="1" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="688" spans="1:2" x14ac:dyDescent="0.35">
@@ -11911,18 +11911,18 @@
     </row>
     <row r="689" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A689" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="B689" s="1" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="690" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A690" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="B690" s="1" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="691" spans="1:2" x14ac:dyDescent="0.35">
@@ -11967,10 +11967,10 @@
     </row>
     <row r="696" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A696" t="s">
+        <v>1517</v>
+      </c>
+      <c r="B696" s="1" t="s">
         <v>1519</v>
-      </c>
-      <c r="B696" s="1" t="s">
-        <v>1521</v>
       </c>
     </row>
     <row r="697" spans="1:2" x14ac:dyDescent="0.35">
@@ -11991,10 +11991,10 @@
     </row>
     <row r="699" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A699" t="s">
-        <v>1517</v>
+        <v>1515</v>
       </c>
       <c r="B699" s="1" t="s">
-        <v>1520</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="700" spans="1:2" x14ac:dyDescent="0.35">
@@ -12103,10 +12103,10 @@
     </row>
     <row r="713" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A713" t="s">
+        <v>1305</v>
+      </c>
+      <c r="B713" s="1" t="s">
         <v>1307</v>
-      </c>
-      <c r="B713" s="1" t="s">
-        <v>1309</v>
       </c>
     </row>
     <row r="714" spans="1:2" x14ac:dyDescent="0.35">
@@ -12207,58 +12207,58 @@
     </row>
     <row r="726" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A726" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="B726" s="1" t="s">
-        <v>1215</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="727" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A727" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="B727" s="1" t="s">
-        <v>1216</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="728" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A728" t="s">
-        <v>1211</v>
+        <v>1209</v>
       </c>
       <c r="B728" s="1" t="s">
-        <v>1217</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="729" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A729" t="s">
-        <v>1455</v>
+        <v>1453</v>
       </c>
       <c r="B729" s="1" t="s">
-        <v>1456</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="730" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A730" t="s">
+        <v>1461</v>
+      </c>
+      <c r="B730" s="1" t="s">
         <v>1463</v>
-      </c>
-      <c r="B730" s="1" t="s">
-        <v>1465</v>
       </c>
     </row>
     <row r="731" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A731" t="s">
-        <v>1458</v>
+        <v>1456</v>
       </c>
       <c r="B731" s="1" t="s">
-        <v>1461</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="732" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A732" t="s">
+        <v>1462</v>
+      </c>
+      <c r="B732" s="1" t="s">
         <v>1464</v>
-      </c>
-      <c r="B732" s="1" t="s">
-        <v>1466</v>
       </c>
     </row>
     <row r="733" spans="1:2" x14ac:dyDescent="0.35">
@@ -12298,7 +12298,7 @@
         <v>1066</v>
       </c>
       <c r="B737" s="1" t="s">
-        <v>1515</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="738" spans="1:2" x14ac:dyDescent="0.35">
@@ -12327,50 +12327,50 @@
     </row>
     <row r="741" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A741" t="s">
-        <v>1791</v>
+        <v>1781</v>
       </c>
       <c r="B741" s="1" t="s">
-        <v>1798</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="742" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A742" t="s">
-        <v>1792</v>
+        <v>1782</v>
       </c>
       <c r="B742" s="1" t="s">
-        <v>1799</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="743" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A743" t="s">
-        <v>1793</v>
+        <v>1783</v>
       </c>
       <c r="B743" s="1" t="s">
-        <v>1800</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="744" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A744" t="s">
-        <v>1769</v>
+        <v>1759</v>
       </c>
       <c r="B744" s="1" t="s">
-        <v>1784</v>
+        <v>1774</v>
       </c>
     </row>
     <row r="745" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A745" t="s">
-        <v>1771</v>
+        <v>1761</v>
       </c>
       <c r="B745" s="1" t="s">
-        <v>1787</v>
+        <v>1777</v>
       </c>
     </row>
     <row r="746" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A746" t="s">
-        <v>1770</v>
+        <v>1760</v>
       </c>
       <c r="B746" s="1" t="s">
-        <v>1788</v>
+        <v>1778</v>
       </c>
     </row>
     <row r="747" spans="1:2" x14ac:dyDescent="0.35">
@@ -12383,58 +12383,58 @@
     </row>
     <row r="748" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A748" t="s">
-        <v>1311</v>
+        <v>1309</v>
       </c>
       <c r="B748" s="1" t="s">
-        <v>1319</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="749" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A749" t="s">
-        <v>1312</v>
+        <v>1310</v>
       </c>
       <c r="B749" s="1" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="750" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A750" t="s">
-        <v>1313</v>
+        <v>1311</v>
       </c>
       <c r="B750" s="1" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="751" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A751" t="s">
-        <v>1660</v>
+        <v>1654</v>
       </c>
       <c r="B751" s="1" t="s">
-        <v>1682</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="752" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A752" t="s">
-        <v>1661</v>
+        <v>1655</v>
       </c>
       <c r="B752" s="1" t="s">
-        <v>1683</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="753" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A753" t="s">
-        <v>1668</v>
+        <v>1662</v>
       </c>
       <c r="B753" s="1" t="s">
-        <v>1686</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="754" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A754" t="s">
-        <v>1669</v>
+        <v>1663</v>
       </c>
       <c r="B754" s="1" t="s">
-        <v>1690</v>
+        <v>1681</v>
       </c>
     </row>
     <row r="755" spans="1:2" x14ac:dyDescent="0.35">
@@ -12479,26 +12479,26 @@
     </row>
     <row r="760" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A760" t="s">
-        <v>1743</v>
+        <v>1733</v>
       </c>
       <c r="B760" s="1" t="s">
-        <v>1749</v>
+        <v>1739</v>
       </c>
     </row>
     <row r="761" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A761" t="s">
-        <v>1745</v>
+        <v>1735</v>
       </c>
       <c r="B761" s="1" t="s">
-        <v>1750</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="762" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A762" t="s">
-        <v>1744</v>
+        <v>1734</v>
       </c>
       <c r="B762" s="1" t="s">
-        <v>1751</v>
+        <v>1741</v>
       </c>
     </row>
     <row r="763" spans="1:2" x14ac:dyDescent="0.35">
@@ -12743,104 +12743,104 @@
     </row>
     <row r="793" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A793" t="s">
-        <v>1249</v>
+        <v>1247</v>
       </c>
       <c r="B793" s="1" t="s">
-        <v>1244</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="794" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A794" t="s">
-        <v>1250</v>
+        <v>1248</v>
       </c>
       <c r="B794" s="1" t="s">
-        <v>1245</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="795" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A795" t="s">
-        <v>1253</v>
+        <v>1251</v>
       </c>
       <c r="B795" s="1" t="s">
-        <v>1254</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="796" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A796" t="s">
+        <v>1491</v>
+      </c>
+      <c r="B796" s="1" t="s">
         <v>1493</v>
-      </c>
-      <c r="B796" s="1" t="s">
-        <v>1495</v>
       </c>
     </row>
     <row r="797" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A797" t="s">
-        <v>1497</v>
+        <v>1495</v>
       </c>
       <c r="B797" s="1" t="s">
-        <v>1504</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="798" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A798" t="s">
-        <v>1497</v>
+        <v>1495</v>
       </c>
       <c r="B798" s="1" t="s">
-        <v>1502</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="799" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A799" t="s">
-        <v>1498</v>
+        <v>1496</v>
       </c>
       <c r="B799" s="1" t="s">
-        <v>1503</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="800" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A800" t="s">
-        <v>1551</v>
+        <v>1549</v>
       </c>
       <c r="B800" s="1" t="s">
-        <v>1541</v>
+        <v>1539</v>
       </c>
       <c r="C800" s="2" t="s">
-        <v>1545</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="801" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A801" t="s">
-        <v>1552</v>
+        <v>1550</v>
       </c>
       <c r="B801" s="1" t="s">
-        <v>1542</v>
+        <v>1540</v>
       </c>
       <c r="C801" s="2" t="s">
-        <v>1546</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="802" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A802" t="s">
-        <v>1713</v>
+        <v>1704</v>
       </c>
       <c r="B802" s="1" t="s">
-        <v>1737</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="803" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A803" t="s">
-        <v>1714</v>
+        <v>1705</v>
       </c>
       <c r="B803" s="1" t="s">
-        <v>1738</v>
+        <v>1728</v>
       </c>
     </row>
     <row r="804" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A804" t="s">
-        <v>1715</v>
+        <v>1706</v>
       </c>
       <c r="B804" s="1" t="s">
-        <v>1739</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="805" spans="1:3" x14ac:dyDescent="0.35">
@@ -12861,26 +12861,26 @@
     </row>
     <row r="807" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A807" t="s">
-        <v>1528</v>
+        <v>1526</v>
       </c>
       <c r="B807" s="1" t="s">
-        <v>1529</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="808" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A808" t="s">
-        <v>1757</v>
+        <v>1747</v>
       </c>
       <c r="B808" s="1" t="s">
-        <v>1765</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="809" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A809" t="s">
-        <v>1758</v>
+        <v>1748</v>
       </c>
       <c r="B809" s="1" t="s">
-        <v>1766</v>
+        <v>1756</v>
       </c>
     </row>
     <row r="810" spans="1:3" x14ac:dyDescent="0.35">
@@ -12909,26 +12909,26 @@
     </row>
     <row r="813" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A813" t="s">
-        <v>1225</v>
+        <v>1223</v>
       </c>
       <c r="B813" s="1" t="s">
-        <v>1231</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="814" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A814" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="B814" s="1" t="s">
-        <v>1232</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="815" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A815" t="s">
-        <v>1227</v>
+        <v>1225</v>
       </c>
       <c r="B815" s="1" t="s">
-        <v>1233</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="816" spans="1:3" x14ac:dyDescent="0.35">
@@ -12989,26 +12989,26 @@
     </row>
     <row r="823" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A823" t="s">
-        <v>1331</v>
+        <v>1329</v>
       </c>
       <c r="B823" s="1" t="s">
-        <v>1337</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="824" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A824" t="s">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="B824" s="1" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="825" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A825" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
       <c r="B825" s="1" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="826" spans="1:2" x14ac:dyDescent="0.35">
@@ -13093,58 +13093,58 @@
     </row>
     <row r="836" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A836" t="s">
-        <v>1296</v>
+        <v>1294</v>
       </c>
       <c r="B836" s="1" t="s">
-        <v>1299</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="837" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A837" t="s">
-        <v>1297</v>
+        <v>1295</v>
       </c>
       <c r="B837" s="1" t="s">
-        <v>1300</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="838" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A838" t="s">
-        <v>1298</v>
+        <v>1296</v>
       </c>
       <c r="B838" s="1" t="s">
-        <v>1301</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="839" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A839" t="s">
+        <v>1506</v>
+      </c>
+      <c r="B839" s="1" t="s">
         <v>1508</v>
-      </c>
-      <c r="B839" s="1" t="s">
-        <v>1510</v>
       </c>
     </row>
     <row r="840" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A840" t="s">
-        <v>1704</v>
+        <v>1695</v>
       </c>
       <c r="B840" s="1" t="s">
-        <v>1711</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="841" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A841" t="s">
-        <v>1702</v>
+        <v>1693</v>
       </c>
       <c r="B841" s="1" t="s">
-        <v>1709</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="842" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A842" t="s">
-        <v>1703</v>
+        <v>1694</v>
       </c>
       <c r="B842" s="1" t="s">
-        <v>1710</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="843" spans="1:2" x14ac:dyDescent="0.35">
@@ -13173,18 +13173,18 @@
     </row>
     <row r="846" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A846" t="s">
-        <v>1626</v>
+        <v>1620</v>
       </c>
       <c r="B846" s="1" t="s">
-        <v>1635</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="847" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A847" t="s">
-        <v>1627</v>
+        <v>1621</v>
       </c>
       <c r="B847" s="1" t="s">
-        <v>1634</v>
+        <v>1628</v>
       </c>
     </row>
     <row r="848" spans="1:2" x14ac:dyDescent="0.35">
@@ -13213,26 +13213,26 @@
     </row>
     <row r="851" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A851" t="s">
-        <v>1774</v>
+        <v>1764</v>
       </c>
       <c r="B851" s="1" t="s">
-        <v>1785</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="852" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A852" t="s">
-        <v>1776</v>
+        <v>1766</v>
       </c>
       <c r="B852" s="1" t="s">
-        <v>1802</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="853" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A853" t="s">
-        <v>1775</v>
+        <v>1765</v>
       </c>
       <c r="B853" s="1" t="s">
-        <v>1803</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="854" spans="1:2" x14ac:dyDescent="0.35">
@@ -13285,10 +13285,10 @@
     </row>
     <row r="860" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A860" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="B860" s="1" t="s">
-        <v>1348</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="861" spans="1:2" x14ac:dyDescent="0.35">
@@ -13325,90 +13325,90 @@
     </row>
     <row r="865" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A865" t="s">
-        <v>1693</v>
+        <v>1684</v>
       </c>
       <c r="B865" s="1" t="s">
-        <v>1698</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="866" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A866" t="s">
-        <v>1693</v>
+        <v>1684</v>
       </c>
       <c r="B866" s="1" t="s">
-        <v>1691</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="867" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A867" t="s">
-        <v>1694</v>
+        <v>1685</v>
       </c>
       <c r="B867" s="1" t="s">
-        <v>1697</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="868" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A868" t="s">
-        <v>1694</v>
+        <v>1685</v>
       </c>
       <c r="B868" s="1" t="s">
-        <v>1699</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="869" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A869" t="s">
-        <v>1654</v>
+        <v>1648</v>
       </c>
       <c r="B869" s="1" t="s">
-        <v>1676</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="870" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A870" t="s">
-        <v>1655</v>
+        <v>1649</v>
       </c>
       <c r="B870" s="1" t="s">
-        <v>1679</v>
+        <v>1671</v>
       </c>
     </row>
     <row r="871" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A871" t="s">
-        <v>1652</v>
+        <v>1646</v>
       </c>
       <c r="B871" s="1" t="s">
-        <v>1677</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="872" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A872" t="s">
-        <v>1653</v>
+        <v>1647</v>
       </c>
       <c r="B872" s="1" t="s">
-        <v>1678</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="873" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A873" t="s">
-        <v>1351</v>
+        <v>1349</v>
       </c>
       <c r="B873" s="1" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="874" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A874" t="s">
-        <v>1352</v>
+        <v>1350</v>
       </c>
       <c r="B874" s="1" t="s">
-        <v>1361</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="875" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A875" t="s">
-        <v>1353</v>
+        <v>1351</v>
       </c>
       <c r="B875" s="1" t="s">
-        <v>1360</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="876" spans="1:2" x14ac:dyDescent="0.35">
@@ -13445,74 +13445,74 @@
     </row>
     <row r="880" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A880" t="s">
-        <v>1605</v>
+        <v>1599</v>
       </c>
       <c r="B880" s="1" t="s">
-        <v>1616</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="881" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A881" t="s">
-        <v>1604</v>
+        <v>1598</v>
       </c>
       <c r="B881" s="1" t="s">
-        <v>1620</v>
+        <v>1614</v>
       </c>
     </row>
     <row r="882" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A882" t="s">
-        <v>1569</v>
+        <v>1567</v>
       </c>
       <c r="B882" s="1" t="s">
-        <v>1565</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="883" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A883" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
       <c r="B883" s="1" t="s">
-        <v>1564</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="884" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A884" t="s">
-        <v>1566</v>
+        <v>1564</v>
       </c>
       <c r="B884" s="1" t="s">
-        <v>1562</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="885" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A885" t="s">
-        <v>1567</v>
+        <v>1565</v>
       </c>
       <c r="B885" s="1" t="s">
-        <v>1563</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="886" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A886" t="s">
-        <v>1607</v>
+        <v>1601</v>
       </c>
       <c r="B886" s="1" t="s">
-        <v>1617</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="887" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A887" t="s">
-        <v>1606</v>
+        <v>1600</v>
       </c>
       <c r="B887" s="1" t="s">
-        <v>1621</v>
+        <v>1615</v>
       </c>
     </row>
     <row r="888" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A888" t="s">
-        <v>1370</v>
+        <v>1368</v>
       </c>
       <c r="B888" s="1" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="889" spans="1:2" x14ac:dyDescent="0.35">
@@ -13573,34 +13573,34 @@
     </row>
     <row r="896" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A896" t="s">
-        <v>1375</v>
+        <v>1373</v>
       </c>
       <c r="B896" s="1" t="s">
-        <v>1373</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="897" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A897" t="s">
+        <v>1370</v>
+      </c>
+      <c r="B897" s="1" t="s">
         <v>1372</v>
-      </c>
-      <c r="B897" s="1" t="s">
-        <v>1374</v>
       </c>
     </row>
     <row r="898" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A898" t="s">
+        <v>1374</v>
+      </c>
+      <c r="B898" s="1" t="s">
         <v>1376</v>
-      </c>
-      <c r="B898" s="1" t="s">
-        <v>1378</v>
       </c>
     </row>
     <row r="899" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A899" t="s">
+        <v>1375</v>
+      </c>
+      <c r="B899" s="1" t="s">
         <v>1377</v>
-      </c>
-      <c r="B899" s="1" t="s">
-        <v>1379</v>
       </c>
     </row>
     <row r="900" spans="1:3" x14ac:dyDescent="0.35">
@@ -13645,26 +13645,26 @@
     </row>
     <row r="905" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A905" t="s">
-        <v>1779</v>
+        <v>1769</v>
       </c>
       <c r="B905" s="1" t="s">
-        <v>1786</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="906" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A906" t="s">
-        <v>1781</v>
+        <v>1771</v>
       </c>
       <c r="B906" s="1" t="s">
-        <v>1804</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="907" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A907" t="s">
-        <v>1780</v>
+        <v>1770</v>
       </c>
       <c r="B907" s="1" t="s">
-        <v>1805</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="908" spans="1:3" x14ac:dyDescent="0.35">
@@ -13817,34 +13817,34 @@
     </row>
     <row r="922" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A922" t="s">
-        <v>1730</v>
+        <v>1720</v>
       </c>
       <c r="B922" s="1" t="s">
-        <v>1729</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="923" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A923" t="s">
-        <v>1670</v>
+        <v>1664</v>
       </c>
       <c r="B923" s="1" t="s">
-        <v>1671</v>
+        <v>1665</v>
       </c>
     </row>
     <row r="924" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A924" t="s">
-        <v>1755</v>
+        <v>1745</v>
       </c>
       <c r="B924" s="1" t="s">
-        <v>1756</v>
+        <v>1746</v>
       </c>
     </row>
     <row r="925" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A925" t="s">
-        <v>1727</v>
+        <v>1717</v>
       </c>
       <c r="B925" s="1" t="s">
-        <v>1728</v>
+        <v>1718</v>
       </c>
     </row>
     <row r="926" spans="1:3" x14ac:dyDescent="0.35">
@@ -13912,7 +13912,7 @@
         <v>219</v>
       </c>
       <c r="B932" s="1" t="s">
-        <v>1256</v>
+        <v>1254</v>
       </c>
       <c r="C932" s="2" t="s">
         <v>220</v>
@@ -13923,15 +13923,15 @@
         <v>987</v>
       </c>
       <c r="B933" s="1" t="s">
-        <v>1257</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="934" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A934" t="s">
-        <v>1731</v>
+        <v>1721</v>
       </c>
       <c r="B934" s="1" t="s">
-        <v>1732</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="935" spans="1:3" x14ac:dyDescent="0.35">
@@ -14077,10 +14077,10 @@
     </row>
     <row r="950" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A950" t="s">
-        <v>1733</v>
+        <v>1723</v>
       </c>
       <c r="B950" s="1" t="s">
-        <v>1734</v>
+        <v>1724</v>
       </c>
     </row>
     <row r="951" spans="1:3" x14ac:dyDescent="0.35">
@@ -14120,10 +14120,10 @@
     </row>
     <row r="955" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A955" t="s">
-        <v>1725</v>
+        <v>1715</v>
       </c>
       <c r="B955" s="1" t="s">
-        <v>1726</v>
+        <v>1716</v>
       </c>
     </row>
     <row r="956" spans="1:3" x14ac:dyDescent="0.35">
@@ -14237,10 +14237,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>1512</v>
+        <v>1510</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1510</v>
+        <v>1508</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>330</v>
@@ -14248,10 +14248,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>1513</v>
+        <v>1511</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1514</v>
+        <v>1512</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>336</v>
@@ -14270,36 +14270,36 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>1454</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>1455</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>1740</v>
+        <v>1730</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>1504</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>1498</v>
+        <v>1496</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>1503</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>1497</v>
+        <v>1495</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>1502</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -14307,7 +14307,7 @@
         <v>1066</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1515</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -14315,31 +14315,31 @@
         <v>1068</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>1516</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>1499</v>
+        <v>1497</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>1505</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>1500</v>
+        <v>1498</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>1506</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>1501</v>
+        <v>1499</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>1507</v>
+        <v>1505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finalized work on offshore wind
</commit_message>
<xml_diff>
--- a/gui/rebalance_localizations.xlsx
+++ b/gui/rebalance_localizations.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">rebalance_localizations!$A$1:$K$963</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">rebalance_localizations!$A$1:$K$969</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet1!#REF!</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -5492,24 +5492,6 @@
     <t>Provides basic protection for the base. Can be built in multiple layers. Cheap reliable and sturdy.</t>
   </si>
   <si>
-    <t>gui/menu/research/name/offsore_wind_lvl_1</t>
-  </si>
-  <si>
-    <t>gui/menu/research/name/offsore_wind_lvl_2</t>
-  </si>
-  <si>
-    <t>gui/menu/research/description/offsore_wind_lvl_2</t>
-  </si>
-  <si>
-    <t>gui/menu/research/description/offsore_wind_lvl_1</t>
-  </si>
-  <si>
-    <t>gui/hud/building_description/offsore_wind_turbine</t>
-  </si>
-  <si>
-    <t>gui/hud/building_name/offsore_wind_turbine</t>
-  </si>
-  <si>
     <t>Offshore Wind Turbine</t>
   </si>
   <si>
@@ -5523,6 +5505,24 @@
   </si>
   <si>
     <t>Wind turbine plattformed adapted for offshore construction to harness wind power whereever it is. Produces power when the wind blows</t>
+  </si>
+  <si>
+    <t>gui/menu/research/description/offshore_wind_lvl_1</t>
+  </si>
+  <si>
+    <t>gui/menu/research/description/offshore_wind_lvl_2</t>
+  </si>
+  <si>
+    <t>gui/menu/research/name/offshore_wind_lvl_1</t>
+  </si>
+  <si>
+    <t>gui/menu/research/name/offshore_wind_lvl_2</t>
+  </si>
+  <si>
+    <t>gui/hud/building_name/offshore_wind_turbine</t>
+  </si>
+  <si>
+    <t>gui/hud/building_description/offshore_wind_turbine</t>
   </si>
 </sst>
 </file>
@@ -7207,10 +7207,10 @@
     </row>
     <row r="101" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>1826</v>
+        <v>1832</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>1828</v>
+        <v>1823</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8668,10 +8668,10 @@
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>1827</v>
+        <v>1831</v>
       </c>
       <c r="B281" s="1" t="s">
-        <v>1829</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.35">
@@ -10856,18 +10856,18 @@
     </row>
     <row r="553" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A553" t="s">
-        <v>1825</v>
+        <v>1827</v>
       </c>
       <c r="B553" s="1" t="s">
-        <v>1832</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="554" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A554" t="s">
-        <v>1824</v>
+        <v>1828</v>
       </c>
       <c r="B554" s="1" t="s">
-        <v>1832</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="555" spans="1:2" x14ac:dyDescent="0.35">
@@ -12974,18 +12974,18 @@
     </row>
     <row r="817" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A817" t="s">
-        <v>1822</v>
+        <v>1829</v>
       </c>
       <c r="B817" s="1" t="s">
-        <v>1830</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="818" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A818" t="s">
-        <v>1823</v>
+        <v>1830</v>
       </c>
       <c r="B818" s="1" t="s">
-        <v>1831</v>
+        <v>1825</v>
       </c>
     </row>
     <row r="819" spans="1:2" x14ac:dyDescent="0.35">
@@ -14296,9 +14296,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K963">
+  <autoFilter ref="A1:K969">
     <sortState ref="A2:K969">
-      <sortCondition ref="A1:A963"/>
+      <sortCondition ref="A1:A969"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
combined wind energy files
</commit_message>
<xml_diff>
--- a/gui/rebalance_localizations.xlsx
+++ b/gui/rebalance_localizations.xlsx
@@ -5498,12 +5498,6 @@
     <t>Larger wind turbine for offshore wind generation. Produces power when the wind blows</t>
   </si>
   <si>
-    <t>Offsore Wind</t>
-  </si>
-  <si>
-    <t>Offsore Wind 2</t>
-  </si>
-  <si>
     <t>Wind turbine plattformed adapted for offshore construction to harness wind power whereever it is. Produces power when the wind blows</t>
   </si>
   <si>
@@ -5523,6 +5517,12 @@
   </si>
   <si>
     <t>gui/hud/building_description/offshore_wind_turbine</t>
+  </si>
+  <si>
+    <t>Offshore Wind Power</t>
+  </si>
+  <si>
+    <t>Offshore Wind Power 2</t>
   </si>
 </sst>
 </file>
@@ -7207,7 +7207,7 @@
     </row>
     <row r="101" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>1832</v>
+        <v>1830</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>1823</v>
@@ -8668,7 +8668,7 @@
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>1831</v>
+        <v>1829</v>
       </c>
       <c r="B281" s="1" t="s">
         <v>1822</v>
@@ -10856,18 +10856,18 @@
     </row>
     <row r="553" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A553" t="s">
-        <v>1827</v>
+        <v>1825</v>
       </c>
       <c r="B553" s="1" t="s">
-        <v>1826</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="554" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A554" t="s">
-        <v>1828</v>
+        <v>1826</v>
       </c>
       <c r="B554" s="1" t="s">
-        <v>1826</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="555" spans="1:2" x14ac:dyDescent="0.35">
@@ -12974,18 +12974,18 @@
     </row>
     <row r="817" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A817" t="s">
-        <v>1829</v>
+        <v>1827</v>
       </c>
       <c r="B817" s="1" t="s">
-        <v>1824</v>
+        <v>1831</v>
       </c>
     </row>
     <row r="818" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A818" t="s">
-        <v>1830</v>
+        <v>1828</v>
       </c>
       <c r="B818" s="1" t="s">
-        <v>1825</v>
+        <v>1832</v>
       </c>
     </row>
     <row r="819" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
fixed inconsistent naming of underground deposits
</commit_message>
<xml_diff>
--- a/gui/rebalance_localizations.xlsx
+++ b/gui/rebalance_localizations.xlsx
@@ -11002,7 +11002,7 @@
     <t xml:space="preserve">resource_name/ammonium_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Ammonium deep vein</t>
+    <t xml:space="preserve">Ammonium Deep Vein</t>
   </si>
   <si>
     <t xml:space="preserve">Tiefe Ammoniumader</t>
@@ -11062,7 +11062,7 @@
     <t xml:space="preserve">resource_name/carbon_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Carbonium vein</t>
+    <t xml:space="preserve">Carbonium Deep Vein</t>
   </si>
   <si>
     <t xml:space="preserve">Carboniumader</t>
@@ -11098,7 +11098,7 @@
     <t xml:space="preserve">resource_name/cobalt_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Cobalt deep vein</t>
+    <t xml:space="preserve">Cobalt Deep Vein</t>
   </si>
   <si>
     <t xml:space="preserve">Tiefe Kobaltader</t>
@@ -11224,7 +11224,7 @@
     <t xml:space="preserve">resource_name/iron_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Ironium vein</t>
+    <t xml:space="preserve">Ironium Deep Vein</t>
   </si>
   <si>
     <t xml:space="preserve">Ironium-Ader</t>
@@ -11296,7 +11296,7 @@
     <t xml:space="preserve">resource_name/morphium_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Morphium well</t>
+    <t xml:space="preserve">Morphium Well</t>
   </si>
   <si>
     <t xml:space="preserve">Morphium-Quelle</t>
@@ -11308,7 +11308,7 @@
     <t xml:space="preserve">resource_name/mud_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Mud well</t>
+    <t xml:space="preserve">Mud Well</t>
   </si>
   <si>
     <t xml:space="preserve">Schlamm-Quelle</t>
@@ -11344,7 +11344,7 @@
     <t xml:space="preserve">resource_name/nitric_acid_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Nitric acid well</t>
+    <t xml:space="preserve">Nitric Acid Well</t>
   </si>
   <si>
     <t xml:space="preserve">Salpetersäure-Quelle</t>
@@ -11365,7 +11365,7 @@
     <t xml:space="preserve">resource_name/palladium_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Palladium deep vein</t>
+    <t xml:space="preserve">Palladium Deep Vein</t>
   </si>
   <si>
     <t xml:space="preserve">Palladium-Tiefader</t>
@@ -11413,7 +11413,7 @@
     <t xml:space="preserve">resource_name/petroleum_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Petroleum well</t>
+    <t xml:space="preserve">Petroleum Well</t>
   </si>
   <si>
     <t xml:space="preserve">Erdölquelle</t>
@@ -11485,7 +11485,7 @@
     <t xml:space="preserve">resource_name/resin_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Resin well</t>
+    <t xml:space="preserve">Resin Well</t>
   </si>
   <si>
     <t xml:space="preserve">Harzquelle</t>
@@ -11497,7 +11497,7 @@
     <t xml:space="preserve">resource_name/sludge_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Sludge well</t>
+    <t xml:space="preserve">Sludge Well</t>
   </si>
   <si>
     <t xml:space="preserve">Schlammquelle</t>
@@ -11557,7 +11557,7 @@
     <t xml:space="preserve">resource_name/titanium_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Titanium deep vein</t>
+    <t xml:space="preserve">Titanium Deep Vein</t>
   </si>
   <si>
     <t xml:space="preserve">Tiefe Titangader</t>
@@ -11605,7 +11605,7 @@
     <t xml:space="preserve">resource_name/uranium_ore_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Uranium Ore deep vein</t>
+    <t xml:space="preserve">Uranium Ore Deep Vein</t>
   </si>
   <si>
     <t xml:space="preserve">Tiefe Uranerzader</t>
@@ -11629,7 +11629,7 @@
     <t xml:space="preserve">resource_name/water_deepvein</t>
   </si>
   <si>
-    <t xml:space="preserve">Water well</t>
+    <t xml:space="preserve">Water Well</t>
   </si>
   <si>
     <t xml:space="preserve">Wasserquelle</t>

</xml_diff>